<commit_message>
Fill in costs for 9 unmatched Goldin cards per user input
Mantle/Ruth/Gehrig triple: $5,000 cost
WNBA Impeccable case: $3,600 cost
Remaining 7 items: $0 (prior year tax loss writeoff)
Goldin unmatched P&L: +$4,019

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018DHCSLBNAQ9LPqbPT7wV3W
</commit_message>
<xml_diff>
--- a/Inventory/Cross_Platform_PL.xlsx
+++ b/Inventory/Cross_Platform_PL.xlsx
@@ -9498,7 +9498,6 @@
           <t>2023-24 Topps Chrome 1972 Topps Autographs Gold Refractor #TA-VW Victor Wembanyama Signed Rookie Card (#04/50) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr"/>
       <c r="E193" s="2" t="n">
         <v>7123.1</v>
       </c>
@@ -9541,7 +9540,6 @@
           <t>2025-26 Topps Silver Pack '80-81 Chrome Basketball Rookie Autographs Orange Refractor #80CR2-CF Cooper Flagg Signed Rookie Card (#17/25) - PSA MINT 9, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr"/>
       <c r="E194" s="2" t="n">
         <v>4427.5</v>
       </c>
@@ -9584,7 +9582,6 @@
           <t>2018-19 Panini National Treasures Peerless Signatures #PS-KBR Kobe Bryant Signed Card (#03/25) - BGS MINT 9, Beckett 10</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
       <c r="E195" s="2" t="n">
         <v>4025</v>
       </c>
@@ -9627,7 +9624,6 @@
           <t>2015-16 Panini Noir Autographs Color Gold #NC-KBR Kobe Bryant Signed Card (#4/5) - PSA EX-MT 6 - Pop 1</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr"/>
       <c r="E196" s="2" t="n">
         <v>3795</v>
       </c>
@@ -9670,7 +9666,6 @@
           <t>2018 Panini Kaboom! #K-NJ Neymar Jr. - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr"/>
       <c r="E197" s="2" t="n">
         <v>3576.5</v>
       </c>
@@ -9713,7 +9708,6 @@
           <t>2003-04 Upper Deck Top Prospects Signs of Success #SS-LJ LeBron James Signed Rookie Card - BGS MINT 9, Beckett 10</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr"/>
       <c r="E198" s="2" t="n">
         <v>3047.5</v>
       </c>
@@ -9756,7 +9750,6 @@
           <t>2025-26 Topps Chrome Future Stars Autographs Green Refractor #FS-CF Cooper Flagg Signed Rookie Card (#43/99) - PSA MINT 9, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr"/>
       <c r="E199" s="2" t="n">
         <v>2760</v>
       </c>
@@ -9799,7 +9792,6 @@
           <t>2023-24 Bowman U Best of 2023 Autograph Geometric Red Refractor #B23-CC Caitlin Clark Signed Rookie Card (#01/10) - PSA MINT 9, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr"/>
       <c r="E200" s="2" t="n">
         <v>2645</v>
       </c>
@@ -9842,7 +9834,6 @@
           <t>2020-21 Panini Flawless Draft Gem Signatures Ruby #DG-AEW Anthony Edwards Signed Rookie Card (#15/15) - Panini Encased</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
       <c r="E201" s="2" t="n">
         <v>2601.3</v>
       </c>
@@ -9885,7 +9876,6 @@
           <t>2023-24 Topps Chrome UCC Future Stars Autographs SuperFractor #FSA-KM Kobbie Mainoo Signed Card (#1/1) - PSA NM-MT 8</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr"/>
       <c r="E202" s="2" t="n">
         <v>2472.5</v>
       </c>
@@ -9928,7 +9918,6 @@
           <t>2022-23 Bowman U Best of '22 Autographs #BOA-VW Victor Wembanyama Signed Rookie Card - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr"/>
       <c r="E203" s="2" t="n">
         <v>2472.5</v>
       </c>
@@ -9971,7 +9960,6 @@
           <t>2025-26 Topps Chrome Next Stop Signatures Purple Geometric Refractor #NS-CF Cooper Flagg Signed Rookie Card (#68/75) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr"/>
       <c r="E204" s="2" t="n">
         <v>2375.9</v>
       </c>
@@ -10015,7 +10003,6 @@
 </t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
       <c r="E205" s="2" t="n">
         <v>2300</v>
       </c>
@@ -10058,7 +10045,6 @@
           <t>2023-24 Topps Chrome UCC Black Lazer Autograph #BLA-LY Lamine Yamal Signed Rookie Card - PSA MINT 9, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
       <c r="E206" s="2" t="n">
         <v>2242.5</v>
       </c>
@@ -10101,7 +10087,6 @@
           <t>2020-21 Panini One and One Rookie Jersey Autographs Blue #RJA-AED Anthony Edwards Signed Patch Rookie Card (#26/35) - PSA Authentic, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr"/>
       <c r="E207" s="2" t="n">
         <v>2127.5</v>
       </c>
@@ -10145,7 +10130,6 @@
 </t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
       <c r="E208" s="2" t="n">
         <v>2070</v>
       </c>
@@ -10189,7 +10173,6 @@
 </t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
       <c r="E209" s="2" t="n">
         <v>2070</v>
       </c>
@@ -10232,7 +10215,6 @@
           <t>2025 Topps Five Star Golden Graphs Blue #GG-YY Yoshinobu Yamamoto Signed Card (#19/20) - Topps Encased</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr"/>
       <c r="E210" s="2" t="n">
         <v>1851.5</v>
       </c>
@@ -10275,7 +10257,6 @@
           <t>2008 Upper Deck SP Rookie Threads SP Dual Threads #TD-BJ Kobe Bryant/Michael Jordan Relic Card - BGS NM-MT+ 8.5</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr"/>
       <c r="E211" s="2" t="n">
         <v>1841.15</v>
       </c>
@@ -10319,7 +10300,6 @@
 </t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
       <c r="E212" s="2" t="n">
         <v>1840</v>
       </c>
@@ -10362,7 +10342,6 @@
           <t>2023-24 Topps Now Autographs #VW-6A Victor Wembanyama Signed Rookie Card (#47/99) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr"/>
       <c r="E213" s="2" t="n">
         <v>1667.5</v>
       </c>
@@ -10405,7 +10384,6 @@
           <t>2019 Topps Diamond Icons Autographs Gold #DIA-MT Mike Trout Signed Card (#1/1) - BGS GEM MINT 9.5, Beckett 10 - True Gem</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
       <c r="E214" s="2" t="n">
         <v>1610</v>
       </c>
@@ -10448,7 +10426,6 @@
           <t>2023-24 Panini Contenders Optic 1986 Tribute Autographs International Jade #86-LKD Luka Doncic Signed Card (#3/5) - Panini Encased</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr"/>
       <c r="E215" s="2" t="n">
         <v>1493.85</v>
       </c>
@@ -10491,7 +10468,6 @@
           <t>2020-21 Panini National Treasures Treasured Signatures Bronze #TS-LUD Luka Doncic Signed Card (#25/25) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr"/>
       <c r="E216" s="2" t="n">
         <v>1463.95</v>
       </c>
@@ -10534,7 +10510,6 @@
           <t>2024-25 Bowman Chrome U Final Exam Autograph #FEA-CF Cooper Flagg Signed Rookie Card - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr"/>
       <c r="E217" s="2" t="n">
         <v>1449</v>
       </c>
@@ -10577,7 +10552,6 @@
           <t>2022-23 Panini Immaculate Collection Scorers Club Signatures #SCS-LUD Luka Doncic Signed Card (#23/25) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr"/>
       <c r="E218" s="2" t="n">
         <v>1392.65</v>
       </c>
@@ -10620,7 +10594,6 @@
           <t>2021-22 Topps Chrome PSG Autograph Wave Refractor #AU-KM Kylian Mbappe Signed Card (#41/50) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
       <c r="E219" s="2" t="n">
         <v>1389.2</v>
       </c>
@@ -10663,7 +10636,6 @@
           <t>2014-15 Panini Flawless Association Autographs Emerald #AA-GA Giannis Antetokounmpo Signed Card (#1/5) - PSA NM 7</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
       <c r="E220" s="2" t="n">
         <v>1151.15</v>
       </c>
@@ -10706,7 +10678,6 @@
           <t>2023-24 Topps Finest Masters Autograph Red/Black Vapor Geometric Refractor #MA-SC Stephen Curry Signed Card (#01/10) - Topps Sealed</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr"/>
       <c r="E221" s="2" t="n">
         <v>1150</v>
       </c>
@@ -10749,7 +10720,6 @@
           <t>2022-23 Panini Noir Autographed Prime Black and White #ANB-LUD Luka Doncic Signed Card (#17/25) - Panini Encased</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr"/>
       <c r="E222" s="2" t="n">
         <v>1150</v>
       </c>
@@ -10793,7 +10763,6 @@
 </t>
         </is>
       </c>
-      <c r="D223" t="inlineStr"/>
       <c r="E223" s="2" t="n">
         <v>1150</v>
       </c>
@@ -10836,7 +10805,6 @@
           <t>2020-21 Panini National Treasures Rookie Private Signings Association #PSA-AED Anthony Edwards Signed Rookie Card - PSA MINT 9 - Pop 4</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr"/>
       <c r="E224" s="2" t="n">
         <v>1150</v>
       </c>
@@ -10879,7 +10847,6 @@
           <t>2019-20 Panini One and One First-Team Signatures #FT-SCY Stephen Curry Signed Card (#08/25) - BGS MINT 9, Beckett 10 - Pop 3</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr"/>
       <c r="E225" s="2" t="n">
         <v>1122.4</v>
       </c>
@@ -10922,7 +10889,6 @@
           <t>2024-25 Topps Regalia Relic Signatures #RRS-SC Stephen Curry Signed Game-Used Patch Card (#03/15) - Topps Encased</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr"/>
       <c r="E226" s="2" t="n">
         <v>1104</v>
       </c>
@@ -10965,7 +10931,6 @@
           <t>2020-21 Panini One and One Rookie Dual Jersey Autograph #RDJ-AED Anthony Edwards Signed Relic Rookie Card (#90/99) - PSA MINT 9, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr"/>
       <c r="E227" s="2" t="n">
         <v>1092.5</v>
       </c>
@@ -11008,7 +10973,6 @@
           <t>1995-96 Upper Deck 23k Gold 50,000 Print Run Michael Jordan (#12516/50000) - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr"/>
       <c r="E228" s="2" t="n">
         <v>977.5</v>
       </c>
@@ -11051,7 +11015,6 @@
           <t>2020-21 Panini Contenders Optic Veteran Seasons Ticket Autograph Orange #VT-JTA Jayson Tatum Signed Card (#06/15) - PSA GEM MT 10, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
       <c r="E229" s="2" t="n">
         <v>874</v>
       </c>
@@ -11094,7 +11057,6 @@
           <t>2022-23 Panini One And One Precision Rookie Jersey Autographs Ruby '25 Black Box #PRJ-PB5 Paolo Banchero Signed Patch Rookie Card (#1/1) - Panini Encased</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr"/>
       <c r="E230" s="2" t="n">
         <v>868.25</v>
       </c>
@@ -11137,7 +11099,6 @@
           <t>2021-22 Panini Donruss Optic Fast Break Signatures Gold #FB-AEW Anthony Edwards Signed Card (#04/10) - PSA MINT 9 - Pop 3</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr"/>
       <c r="E231" s="2" t="n">
         <v>868.25</v>
       </c>
@@ -11181,7 +11142,6 @@
 </t>
         </is>
       </c>
-      <c r="D232" t="inlineStr"/>
       <c r="E232" s="2" t="n">
         <v>862.5</v>
       </c>
@@ -11224,7 +11184,6 @@
           <t>2024-25 Panini One and One Logoman #LM-CDY Cody Williams Logoman Patch Rookie Card (#2/5) - Panini Encased</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr"/>
       <c r="E233" s="2" t="n">
         <v>833.75</v>
       </c>
@@ -11267,7 +11226,6 @@
           <t>2023-24 Bowman Chrome U 2007-08 Bowman Gold #07B-22 Caitlin Clark Rookie Card (#32/50) - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
       <c r="E234" s="2" t="n">
         <v>829.15</v>
       </c>
@@ -11310,7 +11268,6 @@
           <t>2017-18 Panini Noir Rookie Patch Autograph (RPA) Black and White #303 Jayson Tatum Signed Patch Rookie Card (#05/99) - Panini Encased</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
       <c r="E235" s="2" t="n">
         <v>805</v>
       </c>
@@ -11353,7 +11310,6 @@
           <t>2017-18 Panini Flawless Momentous Autographs Gold #MA-GA Giannis Antetokounmpo Signed Card (#04/10) - Panini Encased</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr"/>
       <c r="E236" s="2" t="n">
         <v>776.25</v>
       </c>
@@ -11396,7 +11352,6 @@
           <t>2017-18 Panini Flawless Premium Ink Signatures #PI-GA Giannis Antetokounmpo Signed Card (#12/25) - BGS GEM MINT 9.5, Beckett 10</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr"/>
       <c r="E237" s="2" t="n">
         <v>776.25</v>
       </c>
@@ -11439,7 +11394,6 @@
           <t>2022-23 Panini Flawless Excellence Signatures '25 Black Box #ES-CHG Chet Holmgren Signed Rookie Card (#1/1) - Panini Encased</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr"/>
       <c r="E238" s="2" t="n">
         <v>776.25</v>
       </c>
@@ -11482,7 +11436,6 @@
           <t>2025-26 Topps All Kings #AK-4 Giannis Antetokounmpo - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr"/>
       <c r="E239" s="2" t="n">
         <v>707.25</v>
       </c>
@@ -11525,7 +11478,6 @@
           <t xml:space="preserve">2023-24 Topps Chrome Sapphire Autograph Red Refractor #CG-TM Tyrese Maxey Signed Card (#5/5) - PSA GEM MT 10 - Pop 1 </t>
         </is>
       </c>
-      <c r="D240" t="inlineStr"/>
       <c r="E240" s="2" t="n">
         <v>633.65</v>
       </c>
@@ -11568,7 +11520,6 @@
           <t>2023-24 Panini Immaculate Collection Immaculate Legends #ILE-YM Yao Ming Signed Card (#31/49) - Panini Encased</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr"/>
       <c r="E241" s="2" t="n">
         <v>575</v>
       </c>
@@ -11611,7 +11562,6 @@
           <t>2019-20 Panini Opulence City of Gold Signatures Gold #CG-NJ Nikola Jokic Signed Card (#10/25) - Panini Encased</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr"/>
       <c r="E242" s="2" t="n">
         <v>575</v>
       </c>
@@ -11654,7 +11604,6 @@
           <t>2011-2012 Upper Deck Exquisite Collection Personal Touch #PTC-VC Vince Carter Signed Card (#01/30) - BGS MINT 9, Beckett 10</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr"/>
       <c r="E243" s="2" t="n">
         <v>575</v>
       </c>
@@ -11697,7 +11646,6 @@
           <t>2025 Topps Chrome Black Autograph Gold Refractor #CBA-PS Paul Skenes Signed Card (#05/50) - PSA NM-MT+ 8.5, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr"/>
       <c r="E244" s="2" t="n">
         <v>517.5</v>
       </c>
@@ -11740,7 +11688,6 @@
           <t>2019-20 Panini One and One First-Team Signatures Blue #FT-FJK Nikola Jokic Signed Card (#08/49) - Panini Encased</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr"/>
       <c r="E245" s="2" t="n">
         <v>517.5</v>
       </c>
@@ -11783,7 +11730,6 @@
           <t>2021-22 Panini Chronicles Hometown Heroes Gold #HHR-CCU Cade Cunningham Signed Rookie Card (#01/10) - Panini Encased</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr"/>
       <c r="E246" s="2" t="n">
         <v>494.5</v>
       </c>
@@ -11826,7 +11772,6 @@
           <t>2023 Topps NPB Chrome Topps 2001 Orange Refractor #01-1 Yoshinobu Yamamoto (#01/25) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr"/>
       <c r="E247" s="2" t="n">
         <v>488.75</v>
       </c>
@@ -11869,7 +11814,6 @@
           <t>2025-26 Topps Chrome Rock Stars #RS-17 Dylan Harper Rookie Card - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr"/>
       <c r="E248" s="2" t="n">
         <v>485.3</v>
       </c>
@@ -11912,7 +11856,6 @@
           <t>2019-20 Panini Prizm Sensational Swatches Prizms Orange Ice #SS-SCU Stephen Curry Signed Relic Card - BGS Authentic Sticker Autograph</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr"/>
       <c r="E249" s="2" t="n">
         <v>485.3</v>
       </c>
@@ -11955,7 +11898,6 @@
           <t>2009-10 Upper Deck SP Game Used 3 Star Swatches #3S-BMJ Kobe Bryant/LeBron James/Oscar Robertson Relic Card (#182/299) - BGS NM-MT 8</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr"/>
       <c r="E250" s="2" t="n">
         <v>440.45</v>
       </c>
@@ -11998,7 +11940,6 @@
           <t>2025 Topps Five Star Pentamerous Penmanship #PP-RS Roki Sasaki Signed Rookie Card (#20/25) - Topps Encased</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr"/>
       <c r="E251" s="2" t="n">
         <v>379.5</v>
       </c>
@@ -12041,7 +11982,6 @@
           <t>2024-25 Panini Instant NIL Autographs #VJED-1 VJ Edgecombe Signed Rookie Card (#08/99) - Panini Encased</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr"/>
       <c r="E252" s="2" t="n">
         <v>373.75</v>
       </c>
@@ -12084,7 +12024,6 @@
           <t>1996-97 Upper Deck Michael Jordan Greater Heights #GH6 Michael Jordan - BGS GEM MINT 9.5</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr"/>
       <c r="E253" s="2" t="n">
         <v>316.25</v>
       </c>
@@ -12127,7 +12066,6 @@
           <t>2024-25 Panini NSCC VIP Gold Color Blast #EH Erling Haaland (#16/44) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr"/>
       <c r="E254" s="2" t="n">
         <v>293.25</v>
       </c>
@@ -12170,7 +12108,6 @@
           <t>2014-15 Panini Flawless Association Autographs Gold #AA-JE Julius Erving Signed Card (#03/10) - BGS NM-MT 8</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr"/>
       <c r="E255" s="2" t="n">
         <v>292.1</v>
       </c>
@@ -12213,7 +12150,6 @@
           <t>2019-20 Panini Immaculate Collection Shadowbox Signatures '25 Black Box #SS-VCT Vince Carter Signed Card (#1/1) - Panini Encased</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr"/>
       <c r="E256" s="2" t="n">
         <v>281.75</v>
       </c>
@@ -12256,7 +12192,6 @@
           <t>2024-25 Panini Flawless Vault Memorabilia #FVM-KAT Karl-Anthony Towns Patch Card (#12/25) - PSA NM-MT 8</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr"/>
       <c r="E257" s="2" t="n">
         <v>247.25</v>
       </c>
@@ -12299,7 +12234,6 @@
           <t>2013-14 Upper Deck All-Time Greats Signatures #ATG-J02 Magic Johnson Signed Card (#16/50) - BGS GEM MINT 9.5</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr"/>
       <c r="E258" s="2" t="n">
         <v>235.75</v>
       </c>
@@ -12342,7 +12276,6 @@
           <t>2020-21 Panini Donruss Optic Signature Series #SS-LBL LaMelo Ball Signed Rookie Card - PSA Authentic, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr"/>
       <c r="E259" s="2" t="n">
         <v>195.5</v>
       </c>
@@ -12385,7 +12318,6 @@
           <t>2022-23 Panini Recon Rookie Recon Signatures Purple #RRS-PBC Paolo Banchero Signed Rookie Card (#12/25) - PSA NM-MT 8, PSA/DNA GEM MT 10</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr"/>
       <c r="E260" s="2" t="n">
         <v>149.5</v>
       </c>
@@ -12428,7 +12360,6 @@
           <t>2025-26 Topps Rise To Stardom Black Rainbow #RTS-3 VJ Edgecombe Rookie Card (#01/10) - PSA NM-MT 8</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr"/>
       <c r="E261" s="2" t="n">
         <v>149.5</v>
       </c>
@@ -12471,7 +12402,6 @@
           <t>2022-23 Topps Finest UCC The Man Blue Refractor #FTM-9 Lionel Messi (#072/150) - PSA MINT 9</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr"/>
       <c r="E262" s="2" t="n">
         <v>138</v>
       </c>
@@ -12514,7 +12444,6 @@
           <t>2012-13 Upper Deck Exquisite Collection Dimensions #D-JE Julius Erving Signed Card</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr"/>
       <c r="E263" s="2" t="n">
         <v>117.3</v>
       </c>
@@ -12557,7 +12486,6 @@
           <t>2022-23 Panini Immaculate Collection Patch Autographs Jersey Number #IPA-RGO Rudy Gobert Signed Relic Card (#06/27) - Panini Encased</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr"/>
       <c r="E264" s="2" t="n">
         <v>27.6</v>
       </c>
@@ -12688,12 +12616,13 @@
           <t>2019 Panini Flawless Triple Legends Sapphire #TL-MRG Mickey Mantle/Babe Ruth/Lou Gehrig Relic Card (#05/15) - PSA GEM MT 10 - Pop 2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" s="2" t="n">
         <v>8051.15</v>
       </c>
       <c r="F2" s="9" t="n"/>
-      <c r="G2" s="15" t="n"/>
+      <c r="G2" s="15" t="n">
+        <v>5000</v>
+      </c>
       <c r="H2" s="3">
         <f>IF(G2&lt;&gt;"",E2-G2,"")</f>
         <v/>
@@ -12715,12 +12644,13 @@
           <t>2025 Panini Impeccable WNBA Basketball Factory-Sealed Hobby Case (3 Boxes) - Possible Paige Bueckers, Hailey Van Lith, Kiki Iriafen Rookie Cards</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" s="2" t="n">
         <v>2876.15</v>
       </c>
       <c r="F3" s="9" t="n"/>
-      <c r="G3" s="15" t="n"/>
+      <c r="G3" s="15" t="n">
+        <v>3600</v>
+      </c>
       <c r="H3" s="3">
         <f>IF(G3&lt;&gt;"",E3-G3,"")</f>
         <v/>
@@ -12742,12 +12672,13 @@
           <t>Feb. 27, 2013 - Stephen Curry Signed Full Ticket - Golden State Warriors vs. New York Knicks - Season Highs of 54 Points and 11 3-Pointers - PSA Authentic</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" s="2" t="n">
         <v>529</v>
       </c>
       <c r="F4" s="9" t="n"/>
-      <c r="G4" s="15" t="n"/>
+      <c r="G4" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H4" s="3">
         <f>IF(G4&lt;&gt;"",E4-G4,"")</f>
         <v/>
@@ -12769,12 +12700,13 @@
           <t>Stephen Curry Signed Trading Card - PSA/DNA Authentic</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" s="2" t="n">
         <v>380.65</v>
       </c>
       <c r="F5" s="9" t="n"/>
-      <c r="G5" s="15" t="n"/>
+      <c r="G5" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H5" s="3">
         <f>IF(G5&lt;&gt;"",E5-G5,"")</f>
         <v/>
@@ -12796,12 +12728,13 @@
           <t>1997-98 Fleer Hoops 23k Gold Basketball Texture Bulls Starting Five - PSA GEM MT 10</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" s="2" t="n">
         <v>330.05</v>
       </c>
       <c r="F6" s="9" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="G6" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H6" s="3">
         <f>IF(G6&lt;&gt;"",E6-G6,"")</f>
         <v/>
@@ -12823,12 +12756,13 @@
           <t>2024-25 Topps Deluxe Manchester United Speak of the Devil Autograph Orange Refractor #SD-ZA Zlatan Ibrahimovic Signed Card (#07/25) - PSA MINT 9 - Pop 4</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" s="2" t="n">
         <v>178.25</v>
       </c>
       <c r="F7" s="9" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="G7" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H7" s="3">
         <f>IF(G7&lt;&gt;"",E7-G7,"")</f>
         <v/>
@@ -12850,12 +12784,13 @@
           <t>Mike Tyson Signed Everlast Boxing Glove - Fiterman Sports</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" s="2" t="n">
         <v>126.5</v>
       </c>
       <c r="F8" s="9" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="G8" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="3">
         <f>IF(G8&lt;&gt;"",E8-G8,"")</f>
         <v/>
@@ -12877,12 +12812,13 @@
           <t>2019-20 Panini One and One Dual Jersey Autographs Purple #DJA-DAF De'Aaron Fox Signed Relic Card (#06/35) - Panini Encased</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" s="2" t="n">
         <v>75.90000000000001</v>
       </c>
       <c r="F9" s="9" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="G9" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="3">
         <f>IF(G9&lt;&gt;"",E9-G9,"")</f>
         <v/>
@@ -12904,12 +12840,13 @@
           <t>Allen Iverson Signed Trading Card - PSA/DNA Authentic</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" s="2" t="n">
         <v>71.3</v>
       </c>
       <c r="F10" s="9" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="G10" s="15" t="n">
+        <v>0</v>
+      </c>
       <c r="H10" s="3">
         <f>IF(G10&lt;&gt;"",E10-G10,"")</f>
         <v/>
@@ -13442,7 +13379,6 @@
       <c r="I83" s="2" t="n"/>
       <c r="J83" s="4" t="n"/>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="D85" s="1" t="n"/>
       <c r="E85" s="3" t="n"/>

</xml_diff>

<commit_message>
Set Whatnot costs at 75% of proceeds per user (Wheelhouse sourcing)
Overrides bad auto-matches on Whatnot Matched (was -$31K, now +$4.4K)
and fills Whatnot Unmatched costs ($10.2K). Total Whatnot P&L: +$7.8K.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018DHCSLBNAQ9LPqbPT7wV3W
</commit_message>
<xml_diff>
--- a/Inventory/Cross_Platform_PL.xlsx
+++ b/Inventory/Cross_Platform_PL.xlsx
@@ -17711,7 +17711,9 @@
       <c r="H2" t="n">
         <v>12</v>
       </c>
-      <c r="I2" s="3" t="n"/>
+      <c r="I2" s="3" t="n">
+        <v>9.56</v>
+      </c>
       <c r="J2" s="2">
         <f>IF(I2&lt;&gt;"",I2,G2)</f>
         <v/>
@@ -17758,7 +17760,9 @@
       <c r="H3" t="n">
         <v>17</v>
       </c>
-      <c r="I3" s="3" t="n"/>
+      <c r="I3" s="3" t="n">
+        <v>49.99</v>
+      </c>
       <c r="J3" s="2">
         <f>IF(I3&lt;&gt;"",I3,G3)</f>
         <v/>
@@ -17805,7 +17809,9 @@
       <c r="H4" t="n">
         <v>17</v>
       </c>
-      <c r="I4" s="3" t="n"/>
+      <c r="I4" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J4" s="2">
         <f>IF(I4&lt;&gt;"",I4,G4)</f>
         <v/>
@@ -17852,7 +17858,9 @@
       <c r="H5" t="n">
         <v>15</v>
       </c>
-      <c r="I5" s="3" t="n"/>
+      <c r="I5" s="3" t="n">
+        <v>12.71</v>
+      </c>
       <c r="J5" s="2">
         <f>IF(I5&lt;&gt;"",I5,G5)</f>
         <v/>
@@ -17899,7 +17907,9 @@
       <c r="H6" t="n">
         <v>28</v>
       </c>
-      <c r="I6" s="3" t="n"/>
+      <c r="I6" s="3" t="n">
+        <v>11.14</v>
+      </c>
       <c r="J6" s="2">
         <f>IF(I6&lt;&gt;"",I6,G6)</f>
         <v/>
@@ -17946,7 +17956,9 @@
       <c r="H7" t="n">
         <v>26</v>
       </c>
-      <c r="I7" s="3" t="n"/>
+      <c r="I7" s="3" t="n">
+        <v>24.53</v>
+      </c>
       <c r="J7" s="2">
         <f>IF(I7&lt;&gt;"",I7,G7)</f>
         <v/>
@@ -17993,7 +18005,9 @@
       <c r="H8" t="n">
         <v>15</v>
       </c>
-      <c r="I8" s="3" t="n"/>
+      <c r="I8" s="3" t="n">
+        <v>23.74</v>
+      </c>
       <c r="J8" s="2">
         <f>IF(I8&lt;&gt;"",I8,G8)</f>
         <v/>
@@ -18040,7 +18054,9 @@
       <c r="H9" t="n">
         <v>19</v>
       </c>
-      <c r="I9" s="3" t="n"/>
+      <c r="I9" s="3" t="n">
+        <v>13.5</v>
+      </c>
       <c r="J9" s="2">
         <f>IF(I9&lt;&gt;"",I9,G9)</f>
         <v/>
@@ -18087,7 +18103,9 @@
       <c r="H10" t="n">
         <v>30</v>
       </c>
-      <c r="I10" s="3" t="n"/>
+      <c r="I10" s="3" t="n">
+        <v>866.25</v>
+      </c>
       <c r="J10" s="2">
         <f>IF(I10&lt;&gt;"",I10,G10)</f>
         <v/>
@@ -18134,7 +18152,9 @@
       <c r="H11" t="n">
         <v>26</v>
       </c>
-      <c r="I11" s="3" t="n"/>
+      <c r="I11" s="3" t="n">
+        <v>11.93</v>
+      </c>
       <c r="J11" s="2">
         <f>IF(I11&lt;&gt;"",I11,G11)</f>
         <v/>
@@ -18181,7 +18201,9 @@
       <c r="H12" t="n">
         <v>19</v>
       </c>
-      <c r="I12" s="3" t="n"/>
+      <c r="I12" s="3" t="n">
+        <v>122.72</v>
+      </c>
       <c r="J12" s="2">
         <f>IF(I12&lt;&gt;"",I12,G12)</f>
         <v/>
@@ -18228,7 +18250,9 @@
       <c r="H13" t="n">
         <v>29</v>
       </c>
-      <c r="I13" s="3" t="n"/>
+      <c r="I13" s="3" t="n">
+        <v>1485</v>
+      </c>
       <c r="J13" s="2">
         <f>IF(I13&lt;&gt;"",I13,G13)</f>
         <v/>
@@ -18275,7 +18299,9 @@
       <c r="H14" t="n">
         <v>30</v>
       </c>
-      <c r="I14" s="3" t="n"/>
+      <c r="I14" s="3" t="n">
+        <v>297</v>
+      </c>
       <c r="J14" s="2">
         <f>IF(I14&lt;&gt;"",I14,G14)</f>
         <v/>
@@ -18322,7 +18348,9 @@
       <c r="H15" t="n">
         <v>23</v>
       </c>
-      <c r="I15" s="3" t="n"/>
+      <c r="I15" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="J15" s="2">
         <f>IF(I15&lt;&gt;"",I15,G15)</f>
         <v/>
@@ -18369,7 +18397,9 @@
       <c r="H16" t="n">
         <v>19</v>
       </c>
-      <c r="I16" s="3" t="n"/>
+      <c r="I16" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="J16" s="2">
         <f>IF(I16&lt;&gt;"",I16,G16)</f>
         <v/>
@@ -18416,7 +18446,9 @@
       <c r="H17" t="n">
         <v>28</v>
       </c>
-      <c r="I17" s="3" t="n"/>
+      <c r="I17" s="3" t="n">
+        <v>189.75</v>
+      </c>
       <c r="J17" s="2">
         <f>IF(I17&lt;&gt;"",I17,G17)</f>
         <v/>
@@ -18463,7 +18495,9 @@
       <c r="H18" t="n">
         <v>30</v>
       </c>
-      <c r="I18" s="3" t="n"/>
+      <c r="I18" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J18" s="2">
         <f>IF(I18&lt;&gt;"",I18,G18)</f>
         <v/>
@@ -18510,7 +18544,9 @@
       <c r="H19" t="n">
         <v>32</v>
       </c>
-      <c r="I19" s="3" t="n"/>
+      <c r="I19" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J19" s="2">
         <f>IF(I19&lt;&gt;"",I19,G19)</f>
         <v/>
@@ -18557,7 +18593,9 @@
       <c r="H20" t="n">
         <v>34</v>
       </c>
-      <c r="I20" s="3" t="n"/>
+      <c r="I20" s="3" t="n">
+        <v>11.02</v>
+      </c>
       <c r="J20" s="2">
         <f>IF(I20&lt;&gt;"",I20,G20)</f>
         <v/>
@@ -18604,7 +18642,9 @@
       <c r="H21" t="n">
         <v>25</v>
       </c>
-      <c r="I21" s="3" t="n"/>
+      <c r="I21" s="3" t="n">
+        <v>142.88</v>
+      </c>
       <c r="J21" s="2">
         <f>IF(I21&lt;&gt;"",I21,G21)</f>
         <v/>
@@ -18651,7 +18691,9 @@
       <c r="H22" t="n">
         <v>25</v>
       </c>
-      <c r="I22" s="3" t="n"/>
+      <c r="I22" s="3" t="n">
+        <v>228.75</v>
+      </c>
       <c r="J22" s="2">
         <f>IF(I22&lt;&gt;"",I22,G22)</f>
         <v/>
@@ -18698,7 +18740,9 @@
       <c r="H23" t="n">
         <v>21</v>
       </c>
-      <c r="I23" s="3" t="n"/>
+      <c r="I23" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J23" s="2">
         <f>IF(I23&lt;&gt;"",I23,G23)</f>
         <v/>
@@ -18745,7 +18789,9 @@
       <c r="H24" t="n">
         <v>26</v>
       </c>
-      <c r="I24" s="3" t="n"/>
+      <c r="I24" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="J24" s="2">
         <f>IF(I24&lt;&gt;"",I24,G24)</f>
         <v/>
@@ -18792,7 +18838,9 @@
       <c r="H25" t="n">
         <v>25</v>
       </c>
-      <c r="I25" s="3" t="n"/>
+      <c r="I25" s="3" t="n">
+        <v>150.94</v>
+      </c>
       <c r="J25" s="2">
         <f>IF(I25&lt;&gt;"",I25,G25)</f>
         <v/>
@@ -18839,7 +18887,9 @@
       <c r="H26" t="n">
         <v>22</v>
       </c>
-      <c r="I26" s="3" t="n"/>
+      <c r="I26" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J26" s="2">
         <f>IF(I26&lt;&gt;"",I26,G26)</f>
         <v/>
@@ -18886,7 +18936,9 @@
       <c r="H27" t="n">
         <v>17</v>
       </c>
-      <c r="I27" s="3" t="n"/>
+      <c r="I27" s="3" t="n">
+        <v>3.26</v>
+      </c>
       <c r="J27" s="2">
         <f>IF(I27&lt;&gt;"",I27,G27)</f>
         <v/>
@@ -18933,7 +18985,9 @@
       <c r="H28" t="n">
         <v>17</v>
       </c>
-      <c r="I28" s="3" t="n"/>
+      <c r="I28" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J28" s="2">
         <f>IF(I28&lt;&gt;"",I28,G28)</f>
         <v/>
@@ -18980,7 +19034,9 @@
       <c r="H29" t="n">
         <v>15</v>
       </c>
-      <c r="I29" s="3" t="n"/>
+      <c r="I29" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J29" s="2">
         <f>IF(I29&lt;&gt;"",I29,G29)</f>
         <v/>
@@ -19027,7 +19083,9 @@
       <c r="H30" t="n">
         <v>26</v>
       </c>
-      <c r="I30" s="3" t="n"/>
+      <c r="I30" s="3" t="n">
+        <v>20.59</v>
+      </c>
       <c r="J30" s="2">
         <f>IF(I30&lt;&gt;"",I30,G30)</f>
         <v/>
@@ -19074,7 +19132,9 @@
       <c r="H31" t="n">
         <v>26</v>
       </c>
-      <c r="I31" s="3" t="n"/>
+      <c r="I31" s="3" t="n">
+        <v>16.65</v>
+      </c>
       <c r="J31" s="2">
         <f>IF(I31&lt;&gt;"",I31,G31)</f>
         <v/>
@@ -19121,7 +19181,9 @@
       <c r="H32" t="n">
         <v>21</v>
       </c>
-      <c r="I32" s="3" t="n"/>
+      <c r="I32" s="3" t="n">
+        <v>63.86</v>
+      </c>
       <c r="J32" s="2">
         <f>IF(I32&lt;&gt;"",I32,G32)</f>
         <v/>
@@ -19168,7 +19230,9 @@
       <c r="H33" t="n">
         <v>28</v>
       </c>
-      <c r="I33" s="3" t="n"/>
+      <c r="I33" s="3" t="n">
+        <v>24.41</v>
+      </c>
       <c r="J33" s="2">
         <f>IF(I33&lt;&gt;"",I33,G33)</f>
         <v/>
@@ -19215,7 +19279,9 @@
       <c r="H34" t="n">
         <v>21</v>
       </c>
-      <c r="I34" s="3" t="n"/>
+      <c r="I34" s="3" t="n">
+        <v>118.69</v>
+      </c>
       <c r="J34" s="2">
         <f>IF(I34&lt;&gt;"",I34,G34)</f>
         <v/>
@@ -19262,7 +19328,9 @@
       <c r="H35" t="n">
         <v>28</v>
       </c>
-      <c r="I35" s="3" t="n"/>
+      <c r="I35" s="3" t="n">
+        <v>28.35</v>
+      </c>
       <c r="J35" s="2">
         <f>IF(I35&lt;&gt;"",I35,G35)</f>
         <v/>
@@ -19309,7 +19377,9 @@
       <c r="H36" t="n">
         <v>22</v>
       </c>
-      <c r="I36" s="3" t="n"/>
+      <c r="I36" s="3" t="n">
+        <v>41.92</v>
+      </c>
       <c r="J36" s="2">
         <f>IF(I36&lt;&gt;"",I36,G36)</f>
         <v/>
@@ -19356,7 +19426,9 @@
       <c r="H37" t="n">
         <v>24</v>
       </c>
-      <c r="I37" s="3" t="n"/>
+      <c r="I37" s="3" t="n">
+        <v>44.51</v>
+      </c>
       <c r="J37" s="2">
         <f>IF(I37&lt;&gt;"",I37,G37)</f>
         <v/>
@@ -19403,7 +19475,9 @@
       <c r="H38" t="n">
         <v>22</v>
       </c>
-      <c r="I38" s="3" t="n"/>
+      <c r="I38" s="3" t="n">
+        <v>53.21</v>
+      </c>
       <c r="J38" s="2">
         <f>IF(I38&lt;&gt;"",I38,G38)</f>
         <v/>
@@ -19450,7 +19524,9 @@
       <c r="H39" t="n">
         <v>22</v>
       </c>
-      <c r="I39" s="3" t="n"/>
+      <c r="I39" s="3" t="n">
+        <v>598.13</v>
+      </c>
       <c r="J39" s="2">
         <f>IF(I39&lt;&gt;"",I39,G39)</f>
         <v/>
@@ -19497,7 +19573,9 @@
       <c r="H40" t="n">
         <v>28</v>
       </c>
-      <c r="I40" s="3" t="n"/>
+      <c r="I40" s="3" t="n">
+        <v>54.19</v>
+      </c>
       <c r="J40" s="2">
         <f>IF(I40&lt;&gt;"",I40,G40)</f>
         <v/>
@@ -19544,7 +19622,9 @@
       <c r="H41" t="n">
         <v>25</v>
       </c>
-      <c r="I41" s="3" t="n"/>
+      <c r="I41" s="3" t="n">
+        <v>26.88</v>
+      </c>
       <c r="J41" s="2">
         <f>IF(I41&lt;&gt;"",I41,G41)</f>
         <v/>
@@ -19591,7 +19671,9 @@
       <c r="H42" t="n">
         <v>28</v>
       </c>
-      <c r="I42" s="3" t="n"/>
+      <c r="I42" s="3" t="n">
+        <v>7.99</v>
+      </c>
       <c r="J42" s="2">
         <f>IF(I42&lt;&gt;"",I42,G42)</f>
         <v/>
@@ -19638,7 +19720,9 @@
       <c r="H43" t="n">
         <v>28</v>
       </c>
-      <c r="I43" s="3" t="n"/>
+      <c r="I43" s="3" t="n">
+        <v>129</v>
+      </c>
       <c r="J43" s="2">
         <f>IF(I43&lt;&gt;"",I43,G43)</f>
         <v/>
@@ -19685,7 +19769,9 @@
       <c r="H44" t="n">
         <v>32</v>
       </c>
-      <c r="I44" s="3" t="n"/>
+      <c r="I44" s="3" t="n">
+        <v>187.5</v>
+      </c>
       <c r="J44" s="2">
         <f>IF(I44&lt;&gt;"",I44,G44)</f>
         <v/>
@@ -19732,7 +19818,9 @@
       <c r="H45" t="n">
         <v>24</v>
       </c>
-      <c r="I45" s="3" t="n"/>
+      <c r="I45" s="3" t="n">
+        <v>90.47</v>
+      </c>
       <c r="J45" s="2">
         <f>IF(I45&lt;&gt;"",I45,G45)</f>
         <v/>
@@ -19779,7 +19867,9 @@
       <c r="H46" t="n">
         <v>17</v>
       </c>
-      <c r="I46" s="3" t="n"/>
+      <c r="I46" s="3" t="n">
+        <v>10.35</v>
+      </c>
       <c r="J46" s="2">
         <f>IF(I46&lt;&gt;"",I46,G46)</f>
         <v/>
@@ -19826,7 +19916,9 @@
       <c r="H47" t="n">
         <v>26</v>
       </c>
-      <c r="I47" s="3" t="n"/>
+      <c r="I47" s="3" t="n">
+        <v>106.59</v>
+      </c>
       <c r="J47" s="2">
         <f>IF(I47&lt;&gt;"",I47,G47)</f>
         <v/>
@@ -19873,7 +19965,9 @@
       <c r="H48" t="n">
         <v>16</v>
       </c>
-      <c r="I48" s="3" t="n"/>
+      <c r="I48" s="3" t="n">
+        <v>33.97</v>
+      </c>
       <c r="J48" s="2">
         <f>IF(I48&lt;&gt;"",I48,G48)</f>
         <v/>
@@ -19920,7 +20014,9 @@
       <c r="H49" t="n">
         <v>12</v>
       </c>
-      <c r="I49" s="3" t="n"/>
+      <c r="I49" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="J49" s="2">
         <f>IF(I49&lt;&gt;"",I49,G49)</f>
         <v/>
@@ -19967,7 +20063,9 @@
       <c r="H50" t="n">
         <v>24</v>
       </c>
-      <c r="I50" s="3" t="n"/>
+      <c r="I50" s="3" t="n">
+        <v>120.94</v>
+      </c>
       <c r="J50" s="2">
         <f>IF(I50&lt;&gt;"",I50,G50)</f>
         <v/>
@@ -20014,7 +20112,9 @@
       <c r="H51" t="n">
         <v>23</v>
       </c>
-      <c r="I51" s="3" t="n"/>
+      <c r="I51" s="3" t="n">
+        <v>41.29</v>
+      </c>
       <c r="J51" s="2">
         <f>IF(I51&lt;&gt;"",I51,G51)</f>
         <v/>
@@ -20061,7 +20161,9 @@
       <c r="H52" t="n">
         <v>21</v>
       </c>
-      <c r="I52" s="3" t="n"/>
+      <c r="I52" s="3" t="n">
+        <v>171</v>
+      </c>
       <c r="J52" s="2">
         <f>IF(I52&lt;&gt;"",I52,G52)</f>
         <v/>
@@ -20108,7 +20210,9 @@
       <c r="H53" t="n">
         <v>25</v>
       </c>
-      <c r="I53" s="3" t="n"/>
+      <c r="I53" s="3" t="n">
+        <v>162.75</v>
+      </c>
       <c r="J53" s="2">
         <f>IF(I53&lt;&gt;"",I53,G53)</f>
         <v/>
@@ -20155,7 +20259,9 @@
       <c r="H54" t="n">
         <v>28</v>
       </c>
-      <c r="I54" s="3" t="n"/>
+      <c r="I54" s="3" t="n">
+        <v>73.54000000000001</v>
+      </c>
       <c r="J54" s="2">
         <f>IF(I54&lt;&gt;"",I54,G54)</f>
         <v/>
@@ -20202,7 +20308,9 @@
       <c r="H55" t="n">
         <v>29</v>
       </c>
-      <c r="I55" s="3" t="n"/>
+      <c r="I55" s="3" t="n">
+        <v>33.19</v>
+      </c>
       <c r="J55" s="2">
         <f>IF(I55&lt;&gt;"",I55,G55)</f>
         <v/>
@@ -20249,7 +20357,9 @@
       <c r="H56" t="n">
         <v>28</v>
       </c>
-      <c r="I56" s="3" t="n"/>
+      <c r="I56" s="3" t="n">
+        <v>49.99</v>
+      </c>
       <c r="J56" s="2">
         <f>IF(I56&lt;&gt;"",I56,G56)</f>
         <v/>
@@ -20296,7 +20406,9 @@
       <c r="H57" t="n">
         <v>15</v>
       </c>
-      <c r="I57" s="3" t="n"/>
+      <c r="I57" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J57" s="2">
         <f>IF(I57&lt;&gt;"",I57,G57)</f>
         <v/>
@@ -20343,7 +20455,9 @@
       <c r="H58" t="n">
         <v>15</v>
       </c>
-      <c r="I58" s="3" t="n"/>
+      <c r="I58" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="J58" s="2">
         <f>IF(I58&lt;&gt;"",I58,G58)</f>
         <v/>
@@ -20390,7 +20504,9 @@
       <c r="H59" t="n">
         <v>26</v>
       </c>
-      <c r="I59" s="3" t="n"/>
+      <c r="I59" s="3" t="n">
+        <v>41.29</v>
+      </c>
       <c r="J59" s="2">
         <f>IF(I59&lt;&gt;"",I59,G59)</f>
         <v/>
@@ -20437,7 +20553,9 @@
       <c r="H60" t="n">
         <v>28</v>
       </c>
-      <c r="I60" s="3" t="n"/>
+      <c r="I60" s="3" t="n">
+        <v>39.67</v>
+      </c>
       <c r="J60" s="2">
         <f>IF(I60&lt;&gt;"",I60,G60)</f>
         <v/>
@@ -20484,7 +20602,9 @@
       <c r="H61" t="n">
         <v>17</v>
       </c>
-      <c r="I61" s="3" t="n"/>
+      <c r="I61" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="J61" s="2">
         <f>IF(I61&lt;&gt;"",I61,G61)</f>
         <v/>
@@ -20531,7 +20651,9 @@
       <c r="H62" t="n">
         <v>28</v>
       </c>
-      <c r="I62" s="3" t="n"/>
+      <c r="I62" s="3" t="n">
+        <v>60.64</v>
+      </c>
       <c r="J62" s="2">
         <f>IF(I62&lt;&gt;"",I62,G62)</f>
         <v/>
@@ -20578,7 +20700,9 @@
       <c r="H63" t="n">
         <v>30</v>
       </c>
-      <c r="I63" s="3" t="n"/>
+      <c r="I63" s="3" t="n">
+        <v>16.65</v>
+      </c>
       <c r="J63" s="2">
         <f>IF(I63&lt;&gt;"",I63,G63)</f>
         <v/>
@@ -20625,7 +20749,9 @@
       <c r="H64" t="n">
         <v>32</v>
       </c>
-      <c r="I64" s="3" t="n"/>
+      <c r="I64" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="J64" s="2">
         <f>IF(I64&lt;&gt;"",I64,G64)</f>
         <v/>
@@ -20672,7 +20798,9 @@
       <c r="H65" t="n">
         <v>30</v>
       </c>
-      <c r="I65" s="3" t="n"/>
+      <c r="I65" s="3" t="n">
+        <v>50.96</v>
+      </c>
       <c r="J65" s="2">
         <f>IF(I65&lt;&gt;"",I65,G65)</f>
         <v/>
@@ -20719,7 +20847,9 @@
       <c r="H66" t="n">
         <v>34</v>
       </c>
-      <c r="I66" s="3" t="n"/>
+      <c r="I66" s="3" t="n">
+        <v>10.24</v>
+      </c>
       <c r="J66" s="2">
         <f>IF(I66&lt;&gt;"",I66,G66)</f>
         <v/>
@@ -20766,7 +20896,9 @@
       <c r="H67" t="n">
         <v>28</v>
       </c>
-      <c r="I67" s="3" t="n"/>
+      <c r="I67" s="3" t="n">
+        <v>34.76</v>
+      </c>
       <c r="J67" s="2">
         <f>IF(I67&lt;&gt;"",I67,G67)</f>
         <v/>
@@ -20813,7 +20945,9 @@
       <c r="H68" t="n">
         <v>32</v>
       </c>
-      <c r="I68" s="3" t="n"/>
+      <c r="I68" s="3" t="n">
+        <v>72.56</v>
+      </c>
       <c r="J68" s="2">
         <f>IF(I68&lt;&gt;"",I68,G68)</f>
         <v/>
@@ -20860,7 +20994,9 @@
       <c r="H69" t="n">
         <v>23</v>
       </c>
-      <c r="I69" s="3" t="n"/>
+      <c r="I69" s="3" t="n">
+        <v>23.74</v>
+      </c>
       <c r="J69" s="2">
         <f>IF(I69&lt;&gt;"",I69,G69)</f>
         <v/>
@@ -20907,7 +21043,9 @@
       <c r="H70" t="n">
         <v>23</v>
       </c>
-      <c r="I70" s="3" t="n"/>
+      <c r="I70" s="3" t="n">
+        <v>154.97</v>
+      </c>
       <c r="J70" s="2">
         <f>IF(I70&lt;&gt;"",I70,G70)</f>
         <v/>
@@ -20954,7 +21092,9 @@
       <c r="H71" t="n">
         <v>30</v>
       </c>
-      <c r="I71" s="3" t="n"/>
+      <c r="I71" s="3" t="n">
+        <v>75.15000000000001</v>
+      </c>
       <c r="J71" s="2">
         <f>IF(I71&lt;&gt;"",I71,G71)</f>
         <v/>
@@ -21001,7 +21141,9 @@
       <c r="H72" t="n">
         <v>19</v>
       </c>
-      <c r="I72" s="3" t="n"/>
+      <c r="I72" s="3" t="n">
+        <v>122.72</v>
+      </c>
       <c r="J72" s="2">
         <f>IF(I72&lt;&gt;"",I72,G72)</f>
         <v/>
@@ -21048,7 +21190,9 @@
       <c r="H73" t="n">
         <v>23</v>
       </c>
-      <c r="I73" s="3" t="n"/>
+      <c r="I73" s="3" t="n">
+        <v>118.69</v>
+      </c>
       <c r="J73" s="2">
         <f>IF(I73&lt;&gt;"",I73,G73)</f>
         <v/>
@@ -21095,7 +21239,9 @@
       <c r="H74" t="n">
         <v>20</v>
       </c>
-      <c r="I74" s="3" t="n"/>
+      <c r="I74" s="3" t="n">
+        <v>59.03</v>
+      </c>
       <c r="J74" s="2">
         <f>IF(I74&lt;&gt;"",I74,G74)</f>
         <v/>
@@ -21142,7 +21288,9 @@
       <c r="H75" t="n">
         <v>30</v>
       </c>
-      <c r="I75" s="3" t="n"/>
+      <c r="I75" s="3" t="n">
+        <v>41.29</v>
+      </c>
       <c r="J75" s="2">
         <f>IF(I75&lt;&gt;"",I75,G75)</f>
         <v/>
@@ -21189,7 +21337,9 @@
       <c r="H76" t="n">
         <v>26</v>
       </c>
-      <c r="I76" s="3" t="n"/>
+      <c r="I76" s="3" t="n">
+        <v>66.11</v>
+      </c>
       <c r="J76" s="2">
         <f>IF(I76&lt;&gt;"",I76,G76)</f>
         <v/>
@@ -21236,7 +21386,9 @@
       <c r="H77" t="n">
         <v>36</v>
       </c>
-      <c r="I77" s="3" t="n"/>
+      <c r="I77" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J77" s="2">
         <f>IF(I77&lt;&gt;"",I77,G77)</f>
         <v/>
@@ -21283,7 +21435,9 @@
       <c r="H78" t="n">
         <v>28</v>
       </c>
-      <c r="I78" s="3" t="n"/>
+      <c r="I78" s="3" t="n">
+        <v>106.59</v>
+      </c>
       <c r="J78" s="2">
         <f>IF(I78&lt;&gt;"",I78,G78)</f>
         <v/>
@@ -21330,7 +21484,9 @@
       <c r="H79" t="n">
         <v>30</v>
       </c>
-      <c r="I79" s="3" t="n"/>
+      <c r="I79" s="3" t="n">
+        <v>10.35</v>
+      </c>
       <c r="J79" s="2">
         <f>IF(I79&lt;&gt;"",I79,G79)</f>
         <v/>
@@ -21377,7 +21533,9 @@
       <c r="H80" t="n">
         <v>28</v>
       </c>
-      <c r="I80" s="3" t="n"/>
+      <c r="I80" s="3" t="n">
+        <v>10.35</v>
+      </c>
       <c r="J80" s="2">
         <f>IF(I80&lt;&gt;"",I80,G80)</f>
         <v/>
@@ -21424,7 +21582,9 @@
       <c r="H81" t="n">
         <v>26</v>
       </c>
-      <c r="I81" s="3" t="n"/>
+      <c r="I81" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="J81" s="2">
         <f>IF(I81&lt;&gt;"",I81,G81)</f>
         <v/>
@@ -21471,7 +21631,9 @@
       <c r="H82" t="n">
         <v>28</v>
       </c>
-      <c r="I82" s="3" t="n"/>
+      <c r="I82" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J82" s="2">
         <f>IF(I82&lt;&gt;"",I82,G82)</f>
         <v/>
@@ -21518,7 +21680,9 @@
       <c r="H83" t="n">
         <v>16</v>
       </c>
-      <c r="I83" s="3" t="n"/>
+      <c r="I83" s="3" t="n">
+        <v>133.03</v>
+      </c>
       <c r="J83" s="2">
         <f>IF(I83&lt;&gt;"",I83,G83)</f>
         <v/>
@@ -21565,7 +21729,9 @@
       <c r="H84" t="n">
         <v>12</v>
       </c>
-      <c r="I84" s="3" t="n"/>
+      <c r="I84" s="3" t="n">
+        <v>3.26</v>
+      </c>
       <c r="J84" s="2">
         <f>IF(I84&lt;&gt;"",I84,G84)</f>
         <v/>
@@ -21612,7 +21778,9 @@
       <c r="H85" t="n">
         <v>28</v>
       </c>
-      <c r="I85" s="3" t="n"/>
+      <c r="I85" s="3" t="n">
+        <v>28.46</v>
+      </c>
       <c r="J85" s="2">
         <f>IF(I85&lt;&gt;"",I85,G85)</f>
         <v/>
@@ -21659,7 +21827,9 @@
       <c r="H86" t="n">
         <v>24</v>
       </c>
-      <c r="I86" s="3" t="n"/>
+      <c r="I86" s="3" t="n">
+        <v>15.08</v>
+      </c>
       <c r="J86" s="2">
         <f>IF(I86&lt;&gt;"",I86,G86)</f>
         <v/>
@@ -21706,7 +21876,9 @@
       <c r="H87" t="n">
         <v>26</v>
       </c>
-      <c r="I87" s="3" t="n"/>
+      <c r="I87" s="3" t="n">
+        <v>9.56</v>
+      </c>
       <c r="J87" s="2">
         <f>IF(I87&lt;&gt;"",I87,G87)</f>
         <v/>
@@ -21753,7 +21925,9 @@
       <c r="H88" t="n">
         <v>27</v>
       </c>
-      <c r="I88" s="3" t="n"/>
+      <c r="I88" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="J88" s="2">
         <f>IF(I88&lt;&gt;"",I88,G88)</f>
         <v/>
@@ -21800,7 +21974,9 @@
       <c r="H89" t="n">
         <v>24</v>
       </c>
-      <c r="I89" s="3" t="n"/>
+      <c r="I89" s="3" t="n">
+        <v>19.01</v>
+      </c>
       <c r="J89" s="2">
         <f>IF(I89&lt;&gt;"",I89,G89)</f>
         <v/>
@@ -21847,7 +22023,9 @@
       <c r="H90" t="n">
         <v>21</v>
       </c>
-      <c r="I90" s="3" t="n"/>
+      <c r="I90" s="3" t="n">
+        <v>19.8</v>
+      </c>
       <c r="J90" s="2">
         <f>IF(I90&lt;&gt;"",I90,G90)</f>
         <v/>
@@ -21894,7 +22072,9 @@
       <c r="H91" t="n">
         <v>27</v>
       </c>
-      <c r="I91" s="3" t="n"/>
+      <c r="I91" s="3" t="n">
+        <v>7.99</v>
+      </c>
       <c r="J91" s="2">
         <f>IF(I91&lt;&gt;"",I91,G91)</f>
         <v/>
@@ -21941,7 +22121,9 @@
       <c r="H92" t="n">
         <v>27</v>
       </c>
-      <c r="I92" s="3" t="n"/>
+      <c r="I92" s="3" t="n">
+        <v>7.99</v>
+      </c>
       <c r="J92" s="2">
         <f>IF(I92&lt;&gt;"",I92,G92)</f>
         <v/>
@@ -21988,7 +22170,9 @@
       <c r="H93" t="n">
         <v>18</v>
       </c>
-      <c r="I93" s="3" t="n"/>
+      <c r="I93" s="3" t="n">
+        <v>44.51</v>
+      </c>
       <c r="J93" s="2">
         <f>IF(I93&lt;&gt;"",I93,G93)</f>
         <v/>
@@ -22035,7 +22219,9 @@
       <c r="H94" t="n">
         <v>30</v>
       </c>
-      <c r="I94" s="3" t="n"/>
+      <c r="I94" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="J94" s="2">
         <f>IF(I94&lt;&gt;"",I94,G94)</f>
         <v/>
@@ -22082,7 +22268,9 @@
       <c r="H95" t="n">
         <v>23</v>
       </c>
-      <c r="I95" s="3" t="n"/>
+      <c r="I95" s="3" t="n">
+        <v>11.93</v>
+      </c>
       <c r="J95" s="2">
         <f>IF(I95&lt;&gt;"",I95,G95)</f>
         <v/>
@@ -22129,7 +22317,9 @@
       <c r="H96" t="n">
         <v>30</v>
       </c>
-      <c r="I96" s="3" t="n"/>
+      <c r="I96" s="3" t="n">
+        <v>4.84</v>
+      </c>
       <c r="J96" s="2">
         <f>IF(I96&lt;&gt;"",I96,G96)</f>
         <v/>
@@ -22176,7 +22366,9 @@
       <c r="H97" t="n">
         <v>23</v>
       </c>
-      <c r="I97" s="3" t="n"/>
+      <c r="I97" s="3" t="n">
+        <v>82.42</v>
+      </c>
       <c r="J97" s="2">
         <f>IF(I97&lt;&gt;"",I97,G97)</f>
         <v/>
@@ -22223,7 +22415,9 @@
       <c r="H98" t="n">
         <v>28</v>
       </c>
-      <c r="I98" s="3" t="n"/>
+      <c r="I98" s="3" t="n">
+        <v>75.15000000000001</v>
+      </c>
       <c r="J98" s="2">
         <f>IF(I98&lt;&gt;"",I98,G98)</f>
         <v/>
@@ -22270,7 +22464,9 @@
       <c r="H99" t="n">
         <v>24</v>
       </c>
-      <c r="I99" s="3" t="n"/>
+      <c r="I99" s="3" t="n">
+        <v>26.89</v>
+      </c>
       <c r="J99" s="2">
         <f>IF(I99&lt;&gt;"",I99,G99)</f>
         <v/>
@@ -22317,7 +22513,9 @@
       <c r="H100" t="n">
         <v>29</v>
       </c>
-      <c r="I100" s="3" t="n"/>
+      <c r="I100" s="3" t="n">
+        <v>11.93</v>
+      </c>
       <c r="J100" s="2">
         <f>IF(I100&lt;&gt;"",I100,G100)</f>
         <v/>
@@ -22364,7 +22562,9 @@
       <c r="H101" t="n">
         <v>27</v>
       </c>
-      <c r="I101" s="3" t="n"/>
+      <c r="I101" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J101" s="2">
         <f>IF(I101&lt;&gt;"",I101,G101)</f>
         <v/>
@@ -22411,7 +22611,9 @@
       <c r="H102" t="n">
         <v>24</v>
       </c>
-      <c r="I102" s="3" t="n"/>
+      <c r="I102" s="3" t="n">
+        <v>29.25</v>
+      </c>
       <c r="J102" s="2">
         <f>IF(I102&lt;&gt;"",I102,G102)</f>
         <v/>
@@ -22458,7 +22660,9 @@
       <c r="H103" t="n">
         <v>29</v>
       </c>
-      <c r="I103" s="3" t="n"/>
+      <c r="I103" s="3" t="n">
+        <v>14.17</v>
+      </c>
       <c r="J103" s="2">
         <f>IF(I103&lt;&gt;"",I103,G103)</f>
         <v/>
@@ -22505,7 +22709,9 @@
       <c r="H104" t="n">
         <v>27</v>
       </c>
-      <c r="I104" s="3" t="n"/>
+      <c r="I104" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="J104" s="2">
         <f>IF(I104&lt;&gt;"",I104,G104)</f>
         <v/>
@@ -22552,7 +22758,9 @@
       <c r="H105" t="n">
         <v>27</v>
       </c>
-      <c r="I105" s="3" t="n"/>
+      <c r="I105" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="J105" s="2">
         <f>IF(I105&lt;&gt;"",I105,G105)</f>
         <v/>
@@ -22599,7 +22807,9 @@
       <c r="H106" t="n">
         <v>32</v>
       </c>
-      <c r="I106" s="3" t="n"/>
+      <c r="I106" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="J106" s="2">
         <f>IF(I106&lt;&gt;"",I106,G106)</f>
         <v/>
@@ -22646,7 +22856,9 @@
       <c r="H107" t="n">
         <v>30</v>
       </c>
-      <c r="I107" s="3" t="n"/>
+      <c r="I107" s="3" t="n">
+        <v>9.56</v>
+      </c>
       <c r="J107" s="2">
         <f>IF(I107&lt;&gt;"",I107,G107)</f>
         <v/>
@@ -22693,7 +22905,9 @@
       <c r="H108" t="n">
         <v>27</v>
       </c>
-      <c r="I108" s="3" t="n"/>
+      <c r="I108" s="3" t="n">
+        <v>4.84</v>
+      </c>
       <c r="J108" s="2">
         <f>IF(I108&lt;&gt;"",I108,G108)</f>
         <v/>
@@ -22740,7 +22954,9 @@
       <c r="H109" t="n">
         <v>29</v>
       </c>
-      <c r="I109" s="3" t="n"/>
+      <c r="I109" s="3" t="n">
+        <v>14.96</v>
+      </c>
       <c r="J109" s="2">
         <f>IF(I109&lt;&gt;"",I109,G109)</f>
         <v/>
@@ -22787,7 +23003,9 @@
       <c r="H110" t="n">
         <v>30</v>
       </c>
-      <c r="I110" s="3" t="n"/>
+      <c r="I110" s="3" t="n">
+        <v>7.99</v>
+      </c>
       <c r="J110" s="2">
         <f>IF(I110&lt;&gt;"",I110,G110)</f>
         <v/>
@@ -22834,7 +23052,9 @@
       <c r="H111" t="n">
         <v>25</v>
       </c>
-      <c r="I111" s="3" t="n"/>
+      <c r="I111" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J111" s="2">
         <f>IF(I111&lt;&gt;"",I111,G111)</f>
         <v/>
@@ -22881,7 +23101,9 @@
       <c r="H112" t="n">
         <v>25</v>
       </c>
-      <c r="I112" s="3" t="n"/>
+      <c r="I112" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="J112" s="2">
         <f>IF(I112&lt;&gt;"",I112,G112)</f>
         <v/>
@@ -22928,7 +23150,9 @@
       <c r="H113" t="n">
         <v>26</v>
       </c>
-      <c r="I113" s="3" t="n"/>
+      <c r="I113" s="3" t="n">
+        <v>55.8</v>
+      </c>
       <c r="J113" s="2">
         <f>IF(I113&lt;&gt;"",I113,G113)</f>
         <v/>
@@ -22975,7 +23199,9 @@
       <c r="H114" t="n">
         <v>32</v>
       </c>
-      <c r="I114" s="3" t="n"/>
+      <c r="I114" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="J114" s="2">
         <f>IF(I114&lt;&gt;"",I114,G114)</f>
         <v/>
@@ -23022,7 +23248,9 @@
       <c r="H115" t="n">
         <v>34</v>
       </c>
-      <c r="I115" s="3" t="n"/>
+      <c r="I115" s="3" t="n">
+        <v>110.62</v>
+      </c>
       <c r="J115" s="2">
         <f>IF(I115&lt;&gt;"",I115,G115)</f>
         <v/>
@@ -23069,7 +23297,9 @@
       <c r="H116" t="n">
         <v>30</v>
       </c>
-      <c r="I116" s="3" t="n"/>
+      <c r="I116" s="3" t="n">
+        <v>8.77</v>
+      </c>
       <c r="J116" s="2">
         <f>IF(I116&lt;&gt;"",I116,G116)</f>
         <v/>
@@ -23116,7 +23346,9 @@
       <c r="H117" t="n">
         <v>26</v>
       </c>
-      <c r="I117" s="3" t="n"/>
+      <c r="I117" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="J117" s="2">
         <f>IF(I117&lt;&gt;"",I117,G117)</f>
         <v/>
@@ -23163,7 +23395,9 @@
       <c r="H118" t="n">
         <v>28</v>
       </c>
-      <c r="I118" s="3" t="n"/>
+      <c r="I118" s="3" t="n">
+        <v>171</v>
+      </c>
       <c r="J118" s="2">
         <f>IF(I118&lt;&gt;"",I118,G118)</f>
         <v/>
@@ -23210,7 +23444,9 @@
       <c r="H119" t="n">
         <v>29</v>
       </c>
-      <c r="I119" s="3" t="n"/>
+      <c r="I119" s="3" t="n">
+        <v>26.1</v>
+      </c>
       <c r="J119" s="2">
         <f>IF(I119&lt;&gt;"",I119,G119)</f>
         <v/>
@@ -23257,7 +23493,9 @@
       <c r="H120" t="n">
         <v>28</v>
       </c>
-      <c r="I120" s="3" t="n"/>
+      <c r="I120" s="3" t="n">
+        <v>12.71</v>
+      </c>
       <c r="J120" s="2">
         <f>IF(I120&lt;&gt;"",I120,G120)</f>
         <v/>
@@ -23304,7 +23542,9 @@
       <c r="H121" t="n">
         <v>34</v>
       </c>
-      <c r="I121" s="3" t="n"/>
+      <c r="I121" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="J121" s="2">
         <f>IF(I121&lt;&gt;"",I121,G121)</f>
         <v/>
@@ -23351,7 +23591,9 @@
       <c r="H122" t="n">
         <v>27</v>
       </c>
-      <c r="I122" s="3" t="n"/>
+      <c r="I122" s="3" t="n">
+        <v>20.48</v>
+      </c>
       <c r="J122" s="2">
         <f>IF(I122&lt;&gt;"",I122,G122)</f>
         <v/>
@@ -23398,7 +23640,9 @@
       <c r="H123" t="n">
         <v>26</v>
       </c>
-      <c r="I123" s="3" t="n"/>
+      <c r="I123" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J123" s="2">
         <f>IF(I123&lt;&gt;"",I123,G123)</f>
         <v/>
@@ -23445,7 +23689,9 @@
       <c r="H124" t="n">
         <v>25</v>
       </c>
-      <c r="I124" s="3" t="n"/>
+      <c r="I124" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="J124" s="2">
         <f>IF(I124&lt;&gt;"",I124,G124)</f>
         <v/>
@@ -23492,7 +23738,9 @@
       <c r="H125" t="n">
         <v>28</v>
       </c>
-      <c r="I125" s="3" t="n"/>
+      <c r="I125" s="3" t="n">
+        <v>21.38</v>
+      </c>
       <c r="J125" s="2">
         <f>IF(I125&lt;&gt;"",I125,G125)</f>
         <v/>
@@ -23539,7 +23787,9 @@
       <c r="H126" t="n">
         <v>28</v>
       </c>
-      <c r="I126" s="3" t="n"/>
+      <c r="I126" s="3" t="n">
+        <v>126.75</v>
+      </c>
       <c r="J126" s="2">
         <f>IF(I126&lt;&gt;"",I126,G126)</f>
         <v/>
@@ -23586,7 +23836,9 @@
       <c r="H127" t="n">
         <v>32</v>
       </c>
-      <c r="I127" s="3" t="n"/>
+      <c r="I127" s="3" t="n">
+        <v>134.81</v>
+      </c>
       <c r="J127" s="2">
         <f>IF(I127&lt;&gt;"",I127,G127)</f>
         <v/>
@@ -23633,7 +23885,9 @@
       <c r="H128" t="n">
         <v>12</v>
       </c>
-      <c r="I128" s="3" t="n"/>
+      <c r="I128" s="3" t="n">
+        <v>65.47</v>
+      </c>
       <c r="J128" s="2">
         <f>IF(I128&lt;&gt;"",I128,G128)</f>
         <v/>
@@ -23680,7 +23934,9 @@
       <c r="H129" t="n">
         <v>34</v>
       </c>
-      <c r="I129" s="3" t="n"/>
+      <c r="I129" s="3" t="n">
+        <v>65.47</v>
+      </c>
       <c r="J129" s="2">
         <f>IF(I129&lt;&gt;"",I129,G129)</f>
         <v/>
@@ -23727,7 +23983,9 @@
       <c r="H130" t="n">
         <v>17</v>
       </c>
-      <c r="I130" s="3" t="n"/>
+      <c r="I130" s="3" t="n">
+        <v>130.79</v>
+      </c>
       <c r="J130" s="2">
         <f>IF(I130&lt;&gt;"",I130,G130)</f>
         <v/>
@@ -23774,7 +24032,9 @@
       <c r="H131" t="n">
         <v>34</v>
       </c>
-      <c r="I131" s="3" t="n"/>
+      <c r="I131" s="3" t="n">
+        <v>73.54000000000001</v>
+      </c>
       <c r="J131" s="2">
         <f>IF(I131&lt;&gt;"",I131,G131)</f>
         <v/>
@@ -23821,7 +24081,9 @@
       <c r="H132" t="n">
         <v>21</v>
       </c>
-      <c r="I132" s="3" t="n"/>
+      <c r="I132" s="3" t="n">
+        <v>98.54000000000001</v>
+      </c>
       <c r="J132" s="2">
         <f>IF(I132&lt;&gt;"",I132,G132)</f>
         <v/>
@@ -23868,7 +24130,9 @@
       <c r="H133" t="n">
         <v>23</v>
       </c>
-      <c r="I133" s="3" t="n"/>
+      <c r="I133" s="3" t="n">
+        <v>204</v>
+      </c>
       <c r="J133" s="2">
         <f>IF(I133&lt;&gt;"",I133,G133)</f>
         <v/>
@@ -23915,7 +24179,9 @@
       <c r="H134" t="n">
         <v>14</v>
       </c>
-      <c r="I134" s="3" t="n"/>
+      <c r="I134" s="3" t="n">
+        <v>330</v>
+      </c>
       <c r="J134" s="2">
         <f>IF(I134&lt;&gt;"",I134,G134)</f>
         <v/>
@@ -23962,7 +24228,9 @@
       <c r="H135" t="n">
         <v>32</v>
       </c>
-      <c r="I135" s="3" t="n"/>
+      <c r="I135" s="3" t="n">
+        <v>554.63</v>
+      </c>
       <c r="J135" s="2">
         <f>IF(I135&lt;&gt;"",I135,G135)</f>
         <v/>
@@ -24009,7 +24277,9 @@
       <c r="H136" t="n">
         <v>17</v>
       </c>
-      <c r="I136" s="3" t="n"/>
+      <c r="I136" s="3" t="n">
+        <v>598.13</v>
+      </c>
       <c r="J136" s="2">
         <f>IF(I136&lt;&gt;"",I136,G136)</f>
         <v/>
@@ -24056,7 +24326,9 @@
       <c r="H137" t="n">
         <v>29</v>
       </c>
-      <c r="I137" s="3" t="n"/>
+      <c r="I137" s="3" t="n">
+        <v>556.88</v>
+      </c>
       <c r="J137" s="2">
         <f>IF(I137&lt;&gt;"",I137,G137)</f>
         <v/>
@@ -24103,7 +24375,9 @@
       <c r="H138" t="n">
         <v>22</v>
       </c>
-      <c r="I138" s="3" t="n"/>
+      <c r="I138" s="3" t="n">
+        <v>556.88</v>
+      </c>
       <c r="J138" s="2">
         <f>IF(I138&lt;&gt;"",I138,G138)</f>
         <v/>
@@ -24150,7 +24424,9 @@
       <c r="H139" t="n">
         <v>17</v>
       </c>
-      <c r="I139" s="3" t="n"/>
+      <c r="I139" s="3" t="n">
+        <v>595.88</v>
+      </c>
       <c r="J139" s="2">
         <f>IF(I139&lt;&gt;"",I139,G139)</f>
         <v/>
@@ -24197,7 +24473,9 @@
       <c r="H140" t="n">
         <v>14</v>
       </c>
-      <c r="I140" s="3" t="n"/>
+      <c r="I140" s="3" t="n">
+        <v>742.5</v>
+      </c>
       <c r="J140" s="2">
         <f>IF(I140&lt;&gt;"",I140,G140)</f>
         <v/>
@@ -24211,6 +24489,7 @@
         <v/>
       </c>
     </row>
+    <row r="141"/>
     <row r="142">
       <c r="D142" s="1" t="inlineStr">
         <is>
@@ -24325,7 +24604,9 @@
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="3" t="n"/>
+      <c r="H2" s="3" t="n">
+        <v>2145</v>
+      </c>
       <c r="I2" s="2">
         <f>IF(H2&lt;&gt;"",E2-H2,"")</f>
         <v/>
@@ -24360,7 +24641,9 @@
       <c r="G3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="n"/>
+      <c r="H3" s="3" t="n">
+        <v>866.25</v>
+      </c>
       <c r="I3" s="2">
         <f>IF(H3&lt;&gt;"",E3-H3,"")</f>
         <v/>
@@ -24395,7 +24678,9 @@
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="n"/>
+      <c r="H4" s="3" t="n">
+        <v>657.75</v>
+      </c>
       <c r="I4" s="2">
         <f>IF(H4&lt;&gt;"",E4-H4,"")</f>
         <v/>
@@ -24430,7 +24715,9 @@
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="n"/>
+      <c r="H5" s="3" t="n">
+        <v>616.5</v>
+      </c>
       <c r="I5" s="2">
         <f>IF(H5&lt;&gt;"",E5-H5,"")</f>
         <v/>
@@ -24465,7 +24752,9 @@
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="3" t="n"/>
+      <c r="H6" s="3" t="n">
+        <v>577.5</v>
+      </c>
       <c r="I6" s="2">
         <f>IF(H6&lt;&gt;"",E6-H6,"")</f>
         <v/>
@@ -24500,7 +24789,9 @@
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="3" t="n"/>
+      <c r="H7" s="3" t="n">
+        <v>453.75</v>
+      </c>
       <c r="I7" s="2">
         <f>IF(H7&lt;&gt;"",E7-H7,"")</f>
         <v/>
@@ -24535,7 +24826,9 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="3" t="n"/>
+      <c r="H8" s="3" t="n">
+        <v>379.5</v>
+      </c>
       <c r="I8" s="2">
         <f>IF(H8&lt;&gt;"",E8-H8,"")</f>
         <v/>
@@ -24570,7 +24863,9 @@
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="3" t="n"/>
+      <c r="H9" s="3" t="n">
+        <v>261.75</v>
+      </c>
       <c r="I9" s="2">
         <f>IF(H9&lt;&gt;"",E9-H9,"")</f>
         <v/>
@@ -24605,7 +24900,9 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="3" t="n"/>
+      <c r="H10" s="3" t="n">
+        <v>261.75</v>
+      </c>
       <c r="I10" s="2">
         <f>IF(H10&lt;&gt;"",E10-H10,"")</f>
         <v/>
@@ -24640,7 +24937,9 @@
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="3" t="n"/>
+      <c r="H11" s="3" t="n">
+        <v>253.5</v>
+      </c>
       <c r="I11" s="2">
         <f>IF(H11&lt;&gt;"",E11-H11,"")</f>
         <v/>
@@ -24675,7 +24974,9 @@
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="3" t="n"/>
+      <c r="H12" s="3" t="n">
+        <v>228.75</v>
+      </c>
       <c r="I12" s="2">
         <f>IF(H12&lt;&gt;"",E12-H12,"")</f>
         <v/>
@@ -24710,7 +25011,9 @@
       <c r="G13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="3" t="n"/>
+      <c r="H13" s="3" t="n">
+        <v>214.5</v>
+      </c>
       <c r="I13" s="2">
         <f>IF(H13&lt;&gt;"",E13-H13,"")</f>
         <v/>
@@ -24745,7 +25048,9 @@
       <c r="G14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="3" t="n"/>
+      <c r="H14" s="3" t="n">
+        <v>179.25</v>
+      </c>
       <c r="I14" s="2">
         <f>IF(H14&lt;&gt;"",E14-H14,"")</f>
         <v/>
@@ -24780,7 +25085,9 @@
       <c r="G15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="3" t="n"/>
+      <c r="H15" s="3" t="n">
+        <v>173.25</v>
+      </c>
       <c r="I15" s="2">
         <f>IF(H15&lt;&gt;"",E15-H15,"")</f>
         <v/>
@@ -24815,7 +25122,9 @@
       <c r="G16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="3" t="n"/>
+      <c r="H16" s="3" t="n">
+        <v>162.75</v>
+      </c>
       <c r="I16" s="2">
         <f>IF(H16&lt;&gt;"",E16-H16,"")</f>
         <v/>
@@ -24850,7 +25159,9 @@
       <c r="G17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="3" t="n"/>
+      <c r="H17" s="3" t="n">
+        <v>141.09</v>
+      </c>
       <c r="I17" s="2">
         <f>IF(H17&lt;&gt;"",E17-H17,"")</f>
         <v/>
@@ -24885,7 +25196,9 @@
       <c r="G18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="3" t="n"/>
+      <c r="H18" s="3" t="n">
+        <v>133.03</v>
+      </c>
       <c r="I18" s="2">
         <f>IF(H18&lt;&gt;"",E18-H18,"")</f>
         <v/>
@@ -24920,7 +25233,9 @@
       <c r="G19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="3" t="n"/>
+      <c r="H19" s="3" t="n">
+        <v>126.75</v>
+      </c>
       <c r="I19" s="2">
         <f>IF(H19&lt;&gt;"",E19-H19,"")</f>
         <v/>
@@ -24955,7 +25270,9 @@
       <c r="G20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="3" t="n"/>
+      <c r="H20" s="3" t="n">
+        <v>102.56</v>
+      </c>
       <c r="I20" s="2">
         <f>IF(H20&lt;&gt;"",E20-H20,"")</f>
         <v/>
@@ -24990,7 +25307,9 @@
       <c r="G21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="3" t="n"/>
+      <c r="H21" s="3" t="n">
+        <v>98.53</v>
+      </c>
       <c r="I21" s="2">
         <f>IF(H21&lt;&gt;"",E21-H21,"")</f>
         <v/>
@@ -25025,7 +25344,9 @@
       <c r="G22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="3" t="n"/>
+      <c r="H22" s="3" t="n">
+        <v>90.48</v>
+      </c>
       <c r="I22" s="2">
         <f>IF(H22&lt;&gt;"",E22-H22,"")</f>
         <v/>
@@ -25060,7 +25381,9 @@
       <c r="G23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="3" t="n"/>
+      <c r="H23" s="3" t="n">
+        <v>86.44</v>
+      </c>
       <c r="I23" s="2">
         <f>IF(H23&lt;&gt;"",E23-H23,"")</f>
         <v/>
@@ -25095,7 +25418,9 @@
       <c r="G24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="3" t="n"/>
+      <c r="H24" s="3" t="n">
+        <v>78.38</v>
+      </c>
       <c r="I24" s="2">
         <f>IF(H24&lt;&gt;"",E24-H24,"")</f>
         <v/>
@@ -25130,7 +25455,9 @@
       <c r="G25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="3" t="n"/>
+      <c r="H25" s="3" t="n">
+        <v>70.31</v>
+      </c>
       <c r="I25" s="2">
         <f>IF(H25&lt;&gt;"",E25-H25,"")</f>
         <v/>
@@ -25165,7 +25492,9 @@
       <c r="G26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="3" t="n"/>
+      <c r="H26" s="3" t="n">
+        <v>68.7</v>
+      </c>
       <c r="I26" s="2">
         <f>IF(H26&lt;&gt;"",E26-H26,"")</f>
         <v/>
@@ -25200,7 +25529,9 @@
       <c r="G27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="3" t="n"/>
+      <c r="H27" s="3" t="n">
+        <v>68.7</v>
+      </c>
       <c r="I27" s="2">
         <f>IF(H27&lt;&gt;"",E27-H27,"")</f>
         <v/>
@@ -25235,7 +25566,9 @@
       <c r="G28" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="3" t="n"/>
+      <c r="H28" s="3" t="n">
+        <v>68.7</v>
+      </c>
       <c r="I28" s="2">
         <f>IF(H28&lt;&gt;"",E28-H28,"")</f>
         <v/>
@@ -25270,7 +25603,9 @@
       <c r="G29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="3" t="n"/>
+      <c r="H29" s="3" t="n">
+        <v>65.47</v>
+      </c>
       <c r="I29" s="2">
         <f>IF(H29&lt;&gt;"",E29-H29,"")</f>
         <v/>
@@ -25305,7 +25640,9 @@
       <c r="G30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="3" t="n"/>
+      <c r="H30" s="3" t="n">
+        <v>63.86</v>
+      </c>
       <c r="I30" s="2">
         <f>IF(H30&lt;&gt;"",E30-H30,"")</f>
         <v/>
@@ -25340,7 +25677,9 @@
       <c r="G31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="3" t="n"/>
+      <c r="H31" s="3" t="n">
+        <v>59.66</v>
+      </c>
       <c r="I31" s="2">
         <f>IF(H31&lt;&gt;"",E31-H31,"")</f>
         <v/>
@@ -25375,7 +25714,9 @@
       <c r="G32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="3" t="n"/>
+      <c r="H32" s="3" t="n">
+        <v>55.8</v>
+      </c>
       <c r="I32" s="2">
         <f>IF(H32&lt;&gt;"",E32-H32,"")</f>
         <v/>
@@ -25410,7 +25751,9 @@
       <c r="G33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="3" t="n"/>
+      <c r="H33" s="3" t="n">
+        <v>54.19</v>
+      </c>
       <c r="I33" s="2">
         <f>IF(H33&lt;&gt;"",E33-H33,"")</f>
         <v/>
@@ -25445,7 +25788,9 @@
       <c r="G34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="3" t="n"/>
+      <c r="H34" s="3" t="n">
+        <v>52.57</v>
+      </c>
       <c r="I34" s="2">
         <f>IF(H34&lt;&gt;"",E34-H34,"")</f>
         <v/>
@@ -25480,7 +25825,9 @@
       <c r="G35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="3" t="n"/>
+      <c r="H35" s="3" t="n">
+        <v>52.57</v>
+      </c>
       <c r="I35" s="2">
         <f>IF(H35&lt;&gt;"",E35-H35,"")</f>
         <v/>
@@ -25515,7 +25862,9 @@
       <c r="G36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="3" t="n"/>
+      <c r="H36" s="3" t="n">
+        <v>50.96</v>
+      </c>
       <c r="I36" s="2">
         <f>IF(H36&lt;&gt;"",E36-H36,"")</f>
         <v/>
@@ -25550,7 +25899,9 @@
       <c r="G37" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="3" t="n"/>
+      <c r="H37" s="3" t="n">
+        <v>49.99</v>
+      </c>
       <c r="I37" s="2">
         <f>IF(H37&lt;&gt;"",E37-H37,"")</f>
         <v/>
@@ -25585,7 +25936,9 @@
       <c r="G38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="3" t="n"/>
+      <c r="H38" s="3" t="n">
+        <v>49.35</v>
+      </c>
       <c r="I38" s="2">
         <f>IF(H38&lt;&gt;"",E38-H38,"")</f>
         <v/>
@@ -25620,7 +25973,9 @@
       <c r="G39" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="3" t="n"/>
+      <c r="H39" s="3" t="n">
+        <v>48.15</v>
+      </c>
       <c r="I39" s="2">
         <f>IF(H39&lt;&gt;"",E39-H39,"")</f>
         <v/>
@@ -25655,7 +26010,9 @@
       <c r="G40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="3" t="n"/>
+      <c r="H40" s="3" t="n">
+        <v>47.74</v>
+      </c>
       <c r="I40" s="2">
         <f>IF(H40&lt;&gt;"",E40-H40,"")</f>
         <v/>
@@ -25690,7 +26047,9 @@
       <c r="G41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="3" t="n"/>
+      <c r="H41" s="3" t="n">
+        <v>46.12</v>
+      </c>
       <c r="I41" s="2">
         <f>IF(H41&lt;&gt;"",E41-H41,"")</f>
         <v/>
@@ -25725,7 +26084,9 @@
       <c r="G42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="3" t="n"/>
+      <c r="H42" s="3" t="n">
+        <v>39.67</v>
+      </c>
       <c r="I42" s="2">
         <f>IF(H42&lt;&gt;"",E42-H42,"")</f>
         <v/>
@@ -25760,7 +26121,9 @@
       <c r="G43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="3" t="n"/>
+      <c r="H43" s="3" t="n">
+        <v>39.67</v>
+      </c>
       <c r="I43" s="2">
         <f>IF(H43&lt;&gt;"",E43-H43,"")</f>
         <v/>
@@ -25795,7 +26158,9 @@
       <c r="G44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="3" t="n"/>
+      <c r="H44" s="3" t="n">
+        <v>39.67</v>
+      </c>
       <c r="I44" s="2">
         <f>IF(H44&lt;&gt;"",E44-H44,"")</f>
         <v/>
@@ -25830,7 +26195,9 @@
       <c r="G45" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="3" t="n"/>
+      <c r="H45" s="3" t="n">
+        <v>38.06</v>
+      </c>
       <c r="I45" s="2">
         <f>IF(H45&lt;&gt;"",E45-H45,"")</f>
         <v/>
@@ -25865,7 +26232,9 @@
       <c r="G46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="3" t="n"/>
+      <c r="H46" s="3" t="n">
+        <v>36.34</v>
+      </c>
       <c r="I46" s="2">
         <f>IF(H46&lt;&gt;"",E46-H46,"")</f>
         <v/>
@@ -25900,7 +26269,9 @@
       <c r="G47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="3" t="n"/>
+      <c r="H47" s="3" t="n">
+        <v>35.44</v>
+      </c>
       <c r="I47" s="2">
         <f>IF(H47&lt;&gt;"",E47-H47,"")</f>
         <v/>
@@ -25935,7 +26306,9 @@
       <c r="G48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="3" t="n"/>
+      <c r="H48" s="3" t="n">
+        <v>33.97</v>
+      </c>
       <c r="I48" s="2">
         <f>IF(H48&lt;&gt;"",E48-H48,"")</f>
         <v/>
@@ -25970,7 +26343,9 @@
       <c r="G49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="3" t="n"/>
+      <c r="H49" s="3" t="n">
+        <v>33.19</v>
+      </c>
       <c r="I49" s="2">
         <f>IF(H49&lt;&gt;"",E49-H49,"")</f>
         <v/>
@@ -26005,7 +26380,9 @@
       <c r="G50" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="3" t="n"/>
+      <c r="H50" s="3" t="n">
+        <v>33.19</v>
+      </c>
       <c r="I50" s="2">
         <f>IF(H50&lt;&gt;"",E50-H50,"")</f>
         <v/>
@@ -26040,7 +26417,9 @@
       <c r="G51" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="3" t="n"/>
+      <c r="H51" s="3" t="n">
+        <v>32.4</v>
+      </c>
       <c r="I51" s="2">
         <f>IF(H51&lt;&gt;"",E51-H51,"")</f>
         <v/>
@@ -26075,7 +26454,9 @@
       <c r="G52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="3" t="n"/>
+      <c r="H52" s="3" t="n">
+        <v>30.04</v>
+      </c>
       <c r="I52" s="2">
         <f>IF(H52&lt;&gt;"",E52-H52,"")</f>
         <v/>
@@ -26110,7 +26491,9 @@
       <c r="G53" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="3" t="n"/>
+      <c r="H53" s="3" t="n">
+        <v>30.04</v>
+      </c>
       <c r="I53" s="2">
         <f>IF(H53&lt;&gt;"",E53-H53,"")</f>
         <v/>
@@ -26145,7 +26528,9 @@
       <c r="G54" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="3" t="n"/>
+      <c r="H54" s="3" t="n">
+        <v>26.89</v>
+      </c>
       <c r="I54" s="2">
         <f>IF(H54&lt;&gt;"",E54-H54,"")</f>
         <v/>
@@ -26180,7 +26565,9 @@
       <c r="G55" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="3" t="n"/>
+      <c r="H55" s="3" t="n">
+        <v>26.1</v>
+      </c>
       <c r="I55" s="2">
         <f>IF(H55&lt;&gt;"",E55-H55,"")</f>
         <v/>
@@ -26215,7 +26602,9 @@
       <c r="G56" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="3" t="n"/>
+      <c r="H56" s="3" t="n">
+        <v>25.31</v>
+      </c>
       <c r="I56" s="2">
         <f>IF(H56&lt;&gt;"",E56-H56,"")</f>
         <v/>
@@ -26250,7 +26639,9 @@
       <c r="G57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H57" s="3" t="n"/>
+      <c r="H57" s="3" t="n">
+        <v>24.53</v>
+      </c>
       <c r="I57" s="2">
         <f>IF(H57&lt;&gt;"",E57-H57,"")</f>
         <v/>
@@ -26285,7 +26676,9 @@
       <c r="G58" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H58" s="3" t="n"/>
+      <c r="H58" s="3" t="n">
+        <v>24.41</v>
+      </c>
       <c r="I58" s="2">
         <f>IF(H58&lt;&gt;"",E58-H58,"")</f>
         <v/>
@@ -26320,7 +26713,9 @@
       <c r="G59" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H59" s="3" t="n"/>
+      <c r="H59" s="3" t="n">
+        <v>23.74</v>
+      </c>
       <c r="I59" s="2">
         <f>IF(H59&lt;&gt;"",E59-H59,"")</f>
         <v/>
@@ -26355,7 +26750,9 @@
       <c r="G60" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H60" s="3" t="n"/>
+      <c r="H60" s="3" t="n">
+        <v>22.16</v>
+      </c>
       <c r="I60" s="2">
         <f>IF(H60&lt;&gt;"",E60-H60,"")</f>
         <v/>
@@ -26390,7 +26787,9 @@
       <c r="G61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H61" s="3" t="n"/>
+      <c r="H61" s="3" t="n">
+        <v>22.16</v>
+      </c>
       <c r="I61" s="2">
         <f>IF(H61&lt;&gt;"",E61-H61,"")</f>
         <v/>
@@ -26425,7 +26824,9 @@
       <c r="G62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="3" t="n"/>
+      <c r="H62" s="3" t="n">
+        <v>20.59</v>
+      </c>
       <c r="I62" s="2">
         <f>IF(H62&lt;&gt;"",E62-H62,"")</f>
         <v/>
@@ -26460,7 +26861,9 @@
       <c r="G63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="3" t="n"/>
+      <c r="H63" s="3" t="n">
+        <v>20.59</v>
+      </c>
       <c r="I63" s="2">
         <f>IF(H63&lt;&gt;"",E63-H63,"")</f>
         <v/>
@@ -26495,7 +26898,9 @@
       <c r="G64" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H64" s="3" t="n"/>
+      <c r="H64" s="3" t="n">
+        <v>18.23</v>
+      </c>
       <c r="I64" s="2">
         <f>IF(H64&lt;&gt;"",E64-H64,"")</f>
         <v/>
@@ -26530,7 +26935,9 @@
       <c r="G65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H65" s="3" t="n"/>
+      <c r="H65" s="3" t="n">
+        <v>18.23</v>
+      </c>
       <c r="I65" s="2">
         <f>IF(H65&lt;&gt;"",E65-H65,"")</f>
         <v/>
@@ -26565,7 +26972,9 @@
       <c r="G66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H66" s="3" t="n"/>
+      <c r="H66" s="3" t="n">
+        <v>15.08</v>
+      </c>
       <c r="I66" s="2">
         <f>IF(H66&lt;&gt;"",E66-H66,"")</f>
         <v/>
@@ -26600,7 +27009,9 @@
       <c r="G67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H67" s="3" t="n"/>
+      <c r="H67" s="3" t="n">
+        <v>14.29</v>
+      </c>
       <c r="I67" s="2">
         <f>IF(H67&lt;&gt;"",E67-H67,"")</f>
         <v/>
@@ -26635,7 +27046,9 @@
       <c r="G68" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H68" s="3" t="n"/>
+      <c r="H68" s="3" t="n">
+        <v>13.5</v>
+      </c>
       <c r="I68" s="2">
         <f>IF(H68&lt;&gt;"",E68-H68,"")</f>
         <v/>
@@ -26670,7 +27083,9 @@
       <c r="G69" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H69" s="3" t="n"/>
+      <c r="H69" s="3" t="n">
+        <v>13.5</v>
+      </c>
       <c r="I69" s="2">
         <f>IF(H69&lt;&gt;"",E69-H69,"")</f>
         <v/>
@@ -26705,7 +27120,9 @@
       <c r="G70" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H70" s="3" t="n"/>
+      <c r="H70" s="3" t="n">
+        <v>12.71</v>
+      </c>
       <c r="I70" s="2">
         <f>IF(H70&lt;&gt;"",E70-H70,"")</f>
         <v/>
@@ -26740,7 +27157,9 @@
       <c r="G71" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H71" s="3" t="n"/>
+      <c r="H71" s="3" t="n">
+        <v>12.6</v>
+      </c>
       <c r="I71" s="2">
         <f>IF(H71&lt;&gt;"",E71-H71,"")</f>
         <v/>
@@ -26775,7 +27194,9 @@
       <c r="G72" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H72" s="3" t="n"/>
+      <c r="H72" s="3" t="n">
+        <v>11.93</v>
+      </c>
       <c r="I72" s="2">
         <f>IF(H72&lt;&gt;"",E72-H72,"")</f>
         <v/>
@@ -26810,7 +27231,9 @@
       <c r="G73" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H73" s="3" t="n"/>
+      <c r="H73" s="3" t="n">
+        <v>11.14</v>
+      </c>
       <c r="I73" s="2">
         <f>IF(H73&lt;&gt;"",E73-H73,"")</f>
         <v/>
@@ -26845,7 +27268,9 @@
       <c r="G74" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H74" s="3" t="n"/>
+      <c r="H74" s="3" t="n">
+        <v>11.14</v>
+      </c>
       <c r="I74" s="2">
         <f>IF(H74&lt;&gt;"",E74-H74,"")</f>
         <v/>
@@ -26880,7 +27305,9 @@
       <c r="G75" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H75" s="3" t="n"/>
+      <c r="H75" s="3" t="n">
+        <v>10.35</v>
+      </c>
       <c r="I75" s="2">
         <f>IF(H75&lt;&gt;"",E75-H75,"")</f>
         <v/>
@@ -26915,7 +27342,9 @@
       <c r="G76" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H76" s="3" t="n"/>
+      <c r="H76" s="3" t="n">
+        <v>9.56</v>
+      </c>
       <c r="I76" s="2">
         <f>IF(H76&lt;&gt;"",E76-H76,"")</f>
         <v/>
@@ -26950,7 +27379,9 @@
       <c r="G77" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H77" s="3" t="n"/>
+      <c r="H77" s="3" t="n">
+        <v>8.77</v>
+      </c>
       <c r="I77" s="2">
         <f>IF(H77&lt;&gt;"",E77-H77,"")</f>
         <v/>
@@ -26985,7 +27416,9 @@
       <c r="G78" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H78" s="3" t="n"/>
+      <c r="H78" s="3" t="n">
+        <v>7.99</v>
+      </c>
       <c r="I78" s="2">
         <f>IF(H78&lt;&gt;"",E78-H78,"")</f>
         <v/>
@@ -27020,7 +27453,9 @@
       <c r="G79" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H79" s="3" t="n"/>
+      <c r="H79" s="3" t="n">
+        <v>7.2</v>
+      </c>
       <c r="I79" s="2">
         <f>IF(H79&lt;&gt;"",E79-H79,"")</f>
         <v/>
@@ -27055,7 +27490,9 @@
       <c r="G80" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H80" s="3" t="n"/>
+      <c r="H80" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="I80" s="2">
         <f>IF(H80&lt;&gt;"",E80-H80,"")</f>
         <v/>
@@ -27090,7 +27527,9 @@
       <c r="G81" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H81" s="3" t="n"/>
+      <c r="H81" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="I81" s="2">
         <f>IF(H81&lt;&gt;"",E81-H81,"")</f>
         <v/>
@@ -27125,7 +27564,9 @@
       <c r="G82" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H82" s="3" t="n"/>
+      <c r="H82" s="3" t="n">
+        <v>6.41</v>
+      </c>
       <c r="I82" s="2">
         <f>IF(H82&lt;&gt;"",E82-H82,"")</f>
         <v/>
@@ -27160,7 +27601,9 @@
       <c r="G83" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H83" s="3" t="n"/>
+      <c r="H83" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="I83" s="2">
         <f>IF(H83&lt;&gt;"",E83-H83,"")</f>
         <v/>
@@ -27195,7 +27638,9 @@
       <c r="G84" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H84" s="3" t="n"/>
+      <c r="H84" s="3" t="n">
+        <v>5.62</v>
+      </c>
       <c r="I84" s="2">
         <f>IF(H84&lt;&gt;"",E84-H84,"")</f>
         <v/>
@@ -27230,7 +27675,9 @@
       <c r="G85" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H85" s="3" t="n"/>
+      <c r="H85" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I85" s="2">
         <f>IF(H85&lt;&gt;"",E85-H85,"")</f>
         <v/>
@@ -27265,7 +27712,9 @@
       <c r="G86" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H86" s="3" t="n"/>
+      <c r="H86" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I86" s="2">
         <f>IF(H86&lt;&gt;"",E86-H86,"")</f>
         <v/>
@@ -27300,7 +27749,9 @@
       <c r="G87" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H87" s="3" t="n"/>
+      <c r="H87" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I87" s="2">
         <f>IF(H87&lt;&gt;"",E87-H87,"")</f>
         <v/>
@@ -27335,7 +27786,9 @@
       <c r="G88" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H88" s="3" t="n"/>
+      <c r="H88" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I88" s="2">
         <f>IF(H88&lt;&gt;"",E88-H88,"")</f>
         <v/>
@@ -27370,7 +27823,9 @@
       <c r="G89" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H89" s="3" t="n"/>
+      <c r="H89" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I89" s="2">
         <f>IF(H89&lt;&gt;"",E89-H89,"")</f>
         <v/>
@@ -27405,7 +27860,9 @@
       <c r="G90" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H90" s="3" t="n"/>
+      <c r="H90" s="3" t="n">
+        <v>4.05</v>
+      </c>
       <c r="I90" s="2">
         <f>IF(H90&lt;&gt;"",E90-H90,"")</f>
         <v/>
@@ -27440,7 +27897,9 @@
       <c r="G91" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H91" s="3" t="n"/>
+      <c r="H91" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="I91" s="2">
         <f>IF(H91&lt;&gt;"",E91-H91,"")</f>
         <v/>
@@ -27475,7 +27934,9 @@
       <c r="G92" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H92" s="3" t="n"/>
+      <c r="H92" s="3" t="n">
+        <v>2.48</v>
+      </c>
       <c r="I92" s="2">
         <f>IF(H92&lt;&gt;"",E92-H92,"")</f>
         <v/>
@@ -27510,7 +27971,9 @@
       <c r="G93" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H93" s="3" t="n"/>
+      <c r="H93" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="I93" s="2">
         <f>IF(H93&lt;&gt;"",E93-H93,"")</f>
         <v/>
@@ -27545,7 +28008,9 @@
       <c r="G94" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H94" s="3" t="n"/>
+      <c r="H94" s="3" t="n">
+        <v>1.69</v>
+      </c>
       <c r="I94" s="2">
         <f>IF(H94&lt;&gt;"",E94-H94,"")</f>
         <v/>

</xml_diff>

<commit_message>
Fix Whatnot cost basis: 75 cents recovered on the dollar (loss, not gain)
User clarified proceeds = 75% of cost paid, meaning cost = proceeds/0.75.
Whatnot total P&L: -$10,347 (-25%) across 232 sales.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018DHCSLBNAQ9LPqbPT7wV3W
</commit_message>
<xml_diff>
--- a/Inventory/Cross_Platform_PL.xlsx
+++ b/Inventory/Cross_Platform_PL.xlsx
@@ -17712,7 +17712,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>9.56</v>
+        <v>17</v>
       </c>
       <c r="J2" s="2">
         <f>IF(I2&lt;&gt;"",I2,G2)</f>
@@ -17761,7 +17761,7 @@
         <v>17</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>49.99</v>
+        <v>88.87</v>
       </c>
       <c r="J3" s="2">
         <f>IF(I3&lt;&gt;"",I3,G3)</f>
@@ -17810,7 +17810,7 @@
         <v>17</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J4" s="2">
         <f>IF(I4&lt;&gt;"",I4,G4)</f>
@@ -17859,7 +17859,7 @@
         <v>15</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>12.71</v>
+        <v>22.6</v>
       </c>
       <c r="J5" s="2">
         <f>IF(I5&lt;&gt;"",I5,G5)</f>
@@ -17908,7 +17908,7 @@
         <v>28</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>11.14</v>
+        <v>19.8</v>
       </c>
       <c r="J6" s="2">
         <f>IF(I6&lt;&gt;"",I6,G6)</f>
@@ -17957,7 +17957,7 @@
         <v>26</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>24.53</v>
+        <v>43.6</v>
       </c>
       <c r="J7" s="2">
         <f>IF(I7&lt;&gt;"",I7,G7)</f>
@@ -18006,7 +18006,7 @@
         <v>15</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>23.74</v>
+        <v>42.2</v>
       </c>
       <c r="J8" s="2">
         <f>IF(I8&lt;&gt;"",I8,G8)</f>
@@ -18055,7 +18055,7 @@
         <v>19</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>13.5</v>
+        <v>24</v>
       </c>
       <c r="J9" s="2">
         <f>IF(I9&lt;&gt;"",I9,G9)</f>
@@ -18104,7 +18104,7 @@
         <v>30</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>866.25</v>
+        <v>1540</v>
       </c>
       <c r="J10" s="2">
         <f>IF(I10&lt;&gt;"",I10,G10)</f>
@@ -18153,7 +18153,7 @@
         <v>26</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>11.93</v>
+        <v>21.2</v>
       </c>
       <c r="J11" s="2">
         <f>IF(I11&lt;&gt;"",I11,G11)</f>
@@ -18202,7 +18202,7 @@
         <v>19</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>122.72</v>
+        <v>218.17</v>
       </c>
       <c r="J12" s="2">
         <f>IF(I12&lt;&gt;"",I12,G12)</f>
@@ -18251,7 +18251,7 @@
         <v>29</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1485</v>
+        <v>2640</v>
       </c>
       <c r="J13" s="2">
         <f>IF(I13&lt;&gt;"",I13,G13)</f>
@@ -18300,7 +18300,7 @@
         <v>30</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>297</v>
+        <v>528</v>
       </c>
       <c r="J14" s="2">
         <f>IF(I14&lt;&gt;"",I14,G14)</f>
@@ -18349,7 +18349,7 @@
         <v>23</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="J15" s="2">
         <f>IF(I15&lt;&gt;"",I15,G15)</f>
@@ -18398,7 +18398,7 @@
         <v>19</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="J16" s="2">
         <f>IF(I16&lt;&gt;"",I16,G16)</f>
@@ -18447,7 +18447,7 @@
         <v>28</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>189.75</v>
+        <v>337.33</v>
       </c>
       <c r="J17" s="2">
         <f>IF(I17&lt;&gt;"",I17,G17)</f>
@@ -18496,7 +18496,7 @@
         <v>30</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J18" s="2">
         <f>IF(I18&lt;&gt;"",I18,G18)</f>
@@ -18545,7 +18545,7 @@
         <v>32</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J19" s="2">
         <f>IF(I19&lt;&gt;"",I19,G19)</f>
@@ -18594,7 +18594,7 @@
         <v>34</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>11.02</v>
+        <v>19.6</v>
       </c>
       <c r="J20" s="2">
         <f>IF(I20&lt;&gt;"",I20,G20)</f>
@@ -18643,7 +18643,7 @@
         <v>25</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>142.88</v>
+        <v>254</v>
       </c>
       <c r="J21" s="2">
         <f>IF(I21&lt;&gt;"",I21,G21)</f>
@@ -18692,7 +18692,7 @@
         <v>25</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>228.75</v>
+        <v>406.67</v>
       </c>
       <c r="J22" s="2">
         <f>IF(I22&lt;&gt;"",I22,G22)</f>
@@ -18741,7 +18741,7 @@
         <v>21</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="J23" s="2">
         <f>IF(I23&lt;&gt;"",I23,G23)</f>
@@ -18790,7 +18790,7 @@
         <v>26</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="J24" s="2">
         <f>IF(I24&lt;&gt;"",I24,G24)</f>
@@ -18839,7 +18839,7 @@
         <v>25</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>150.94</v>
+        <v>268.33</v>
       </c>
       <c r="J25" s="2">
         <f>IF(I25&lt;&gt;"",I25,G25)</f>
@@ -18888,7 +18888,7 @@
         <v>22</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J26" s="2">
         <f>IF(I26&lt;&gt;"",I26,G26)</f>
@@ -18937,7 +18937,7 @@
         <v>17</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>3.26</v>
+        <v>5.8</v>
       </c>
       <c r="J27" s="2">
         <f>IF(I27&lt;&gt;"",I27,G27)</f>
@@ -18986,7 +18986,7 @@
         <v>17</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="J28" s="2">
         <f>IF(I28&lt;&gt;"",I28,G28)</f>
@@ -19035,7 +19035,7 @@
         <v>15</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="J29" s="2">
         <f>IF(I29&lt;&gt;"",I29,G29)</f>
@@ -19084,7 +19084,7 @@
         <v>26</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>20.59</v>
+        <v>36.6</v>
       </c>
       <c r="J30" s="2">
         <f>IF(I30&lt;&gt;"",I30,G30)</f>
@@ -19133,7 +19133,7 @@
         <v>26</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>16.65</v>
+        <v>29.6</v>
       </c>
       <c r="J31" s="2">
         <f>IF(I31&lt;&gt;"",I31,G31)</f>
@@ -19182,7 +19182,7 @@
         <v>21</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>63.86</v>
+        <v>113.53</v>
       </c>
       <c r="J32" s="2">
         <f>IF(I32&lt;&gt;"",I32,G32)</f>
@@ -19231,7 +19231,7 @@
         <v>28</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>24.41</v>
+        <v>43.4</v>
       </c>
       <c r="J33" s="2">
         <f>IF(I33&lt;&gt;"",I33,G33)</f>
@@ -19280,7 +19280,7 @@
         <v>21</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>118.69</v>
+        <v>211</v>
       </c>
       <c r="J34" s="2">
         <f>IF(I34&lt;&gt;"",I34,G34)</f>
@@ -19329,7 +19329,7 @@
         <v>28</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>28.35</v>
+        <v>50.4</v>
       </c>
       <c r="J35" s="2">
         <f>IF(I35&lt;&gt;"",I35,G35)</f>
@@ -19378,7 +19378,7 @@
         <v>22</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>41.92</v>
+        <v>74.53</v>
       </c>
       <c r="J36" s="2">
         <f>IF(I36&lt;&gt;"",I36,G36)</f>
@@ -19427,7 +19427,7 @@
         <v>24</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>44.51</v>
+        <v>79.13</v>
       </c>
       <c r="J37" s="2">
         <f>IF(I37&lt;&gt;"",I37,G37)</f>
@@ -19476,7 +19476,7 @@
         <v>22</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>53.21</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="J38" s="2">
         <f>IF(I38&lt;&gt;"",I38,G38)</f>
@@ -19525,7 +19525,7 @@
         <v>22</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>598.13</v>
+        <v>1063.33</v>
       </c>
       <c r="J39" s="2">
         <f>IF(I39&lt;&gt;"",I39,G39)</f>
@@ -19574,7 +19574,7 @@
         <v>28</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>54.19</v>
+        <v>96.33</v>
       </c>
       <c r="J40" s="2">
         <f>IF(I40&lt;&gt;"",I40,G40)</f>
@@ -19623,7 +19623,7 @@
         <v>25</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>26.88</v>
+        <v>47.79</v>
       </c>
       <c r="J41" s="2">
         <f>IF(I41&lt;&gt;"",I41,G41)</f>
@@ -19672,7 +19672,7 @@
         <v>28</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>7.99</v>
+        <v>14.2</v>
       </c>
       <c r="J42" s="2">
         <f>IF(I42&lt;&gt;"",I42,G42)</f>
@@ -19721,7 +19721,7 @@
         <v>28</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>129</v>
+        <v>229.33</v>
       </c>
       <c r="J43" s="2">
         <f>IF(I43&lt;&gt;"",I43,G43)</f>
@@ -19770,7 +19770,7 @@
         <v>32</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>187.5</v>
+        <v>333.33</v>
       </c>
       <c r="J44" s="2">
         <f>IF(I44&lt;&gt;"",I44,G44)</f>
@@ -19819,7 +19819,7 @@
         <v>24</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>90.47</v>
+        <v>160.84</v>
       </c>
       <c r="J45" s="2">
         <f>IF(I45&lt;&gt;"",I45,G45)</f>
@@ -19868,7 +19868,7 @@
         <v>17</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>10.35</v>
+        <v>18.4</v>
       </c>
       <c r="J46" s="2">
         <f>IF(I46&lt;&gt;"",I46,G46)</f>
@@ -19917,7 +19917,7 @@
         <v>26</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>106.59</v>
+        <v>189.5</v>
       </c>
       <c r="J47" s="2">
         <f>IF(I47&lt;&gt;"",I47,G47)</f>
@@ -19966,7 +19966,7 @@
         <v>16</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>33.97</v>
+        <v>60.4</v>
       </c>
       <c r="J48" s="2">
         <f>IF(I48&lt;&gt;"",I48,G48)</f>
@@ -20015,7 +20015,7 @@
         <v>12</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="J49" s="2">
         <f>IF(I49&lt;&gt;"",I49,G49)</f>
@@ -20064,7 +20064,7 @@
         <v>24</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>120.94</v>
+        <v>215</v>
       </c>
       <c r="J50" s="2">
         <f>IF(I50&lt;&gt;"",I50,G50)</f>
@@ -20113,7 +20113,7 @@
         <v>23</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>41.29</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J51" s="2">
         <f>IF(I51&lt;&gt;"",I51,G51)</f>
@@ -20162,7 +20162,7 @@
         <v>21</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>171</v>
+        <v>304</v>
       </c>
       <c r="J52" s="2">
         <f>IF(I52&lt;&gt;"",I52,G52)</f>
@@ -20211,7 +20211,7 @@
         <v>25</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>162.75</v>
+        <v>289.33</v>
       </c>
       <c r="J53" s="2">
         <f>IF(I53&lt;&gt;"",I53,G53)</f>
@@ -20260,7 +20260,7 @@
         <v>28</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>73.54000000000001</v>
+        <v>130.73</v>
       </c>
       <c r="J54" s="2">
         <f>IF(I54&lt;&gt;"",I54,G54)</f>
@@ -20309,7 +20309,7 @@
         <v>29</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>33.19</v>
+        <v>59</v>
       </c>
       <c r="J55" s="2">
         <f>IF(I55&lt;&gt;"",I55,G55)</f>
@@ -20358,7 +20358,7 @@
         <v>28</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>49.99</v>
+        <v>88.87</v>
       </c>
       <c r="J56" s="2">
         <f>IF(I56&lt;&gt;"",I56,G56)</f>
@@ -20407,7 +20407,7 @@
         <v>15</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J57" s="2">
         <f>IF(I57&lt;&gt;"",I57,G57)</f>
@@ -20456,7 +20456,7 @@
         <v>15</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="J58" s="2">
         <f>IF(I58&lt;&gt;"",I58,G58)</f>
@@ -20505,7 +20505,7 @@
         <v>26</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>41.29</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J59" s="2">
         <f>IF(I59&lt;&gt;"",I59,G59)</f>
@@ -20554,7 +20554,7 @@
         <v>28</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>39.67</v>
+        <v>70.53</v>
       </c>
       <c r="J60" s="2">
         <f>IF(I60&lt;&gt;"",I60,G60)</f>
@@ -20603,7 +20603,7 @@
         <v>17</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="J61" s="2">
         <f>IF(I61&lt;&gt;"",I61,G61)</f>
@@ -20652,7 +20652,7 @@
         <v>28</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>60.64</v>
+        <v>107.8</v>
       </c>
       <c r="J62" s="2">
         <f>IF(I62&lt;&gt;"",I62,G62)</f>
@@ -20701,7 +20701,7 @@
         <v>30</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>16.65</v>
+        <v>29.6</v>
       </c>
       <c r="J63" s="2">
         <f>IF(I63&lt;&gt;"",I63,G63)</f>
@@ -20750,7 +20750,7 @@
         <v>32</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="J64" s="2">
         <f>IF(I64&lt;&gt;"",I64,G64)</f>
@@ -20799,7 +20799,7 @@
         <v>30</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>50.96</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="J65" s="2">
         <f>IF(I65&lt;&gt;"",I65,G65)</f>
@@ -20848,7 +20848,7 @@
         <v>34</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>10.24</v>
+        <v>18.2</v>
       </c>
       <c r="J66" s="2">
         <f>IF(I66&lt;&gt;"",I66,G66)</f>
@@ -20897,7 +20897,7 @@
         <v>28</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>34.76</v>
+        <v>61.8</v>
       </c>
       <c r="J67" s="2">
         <f>IF(I67&lt;&gt;"",I67,G67)</f>
@@ -20946,7 +20946,7 @@
         <v>32</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>72.56</v>
+        <v>129</v>
       </c>
       <c r="J68" s="2">
         <f>IF(I68&lt;&gt;"",I68,G68)</f>
@@ -20995,7 +20995,7 @@
         <v>23</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>23.74</v>
+        <v>42.2</v>
       </c>
       <c r="J69" s="2">
         <f>IF(I69&lt;&gt;"",I69,G69)</f>
@@ -21044,7 +21044,7 @@
         <v>23</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>154.97</v>
+        <v>275.51</v>
       </c>
       <c r="J70" s="2">
         <f>IF(I70&lt;&gt;"",I70,G70)</f>
@@ -21093,7 +21093,7 @@
         <v>30</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>75.15000000000001</v>
+        <v>133.6</v>
       </c>
       <c r="J71" s="2">
         <f>IF(I71&lt;&gt;"",I71,G71)</f>
@@ -21142,7 +21142,7 @@
         <v>19</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>122.72</v>
+        <v>218.17</v>
       </c>
       <c r="J72" s="2">
         <f>IF(I72&lt;&gt;"",I72,G72)</f>
@@ -21191,7 +21191,7 @@
         <v>23</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>118.69</v>
+        <v>211</v>
       </c>
       <c r="J73" s="2">
         <f>IF(I73&lt;&gt;"",I73,G73)</f>
@@ -21240,7 +21240,7 @@
         <v>20</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>59.03</v>
+        <v>104.93</v>
       </c>
       <c r="J74" s="2">
         <f>IF(I74&lt;&gt;"",I74,G74)</f>
@@ -21289,7 +21289,7 @@
         <v>30</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>41.29</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="J75" s="2">
         <f>IF(I75&lt;&gt;"",I75,G75)</f>
@@ -21338,7 +21338,7 @@
         <v>26</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>66.11</v>
+        <v>117.53</v>
       </c>
       <c r="J76" s="2">
         <f>IF(I76&lt;&gt;"",I76,G76)</f>
@@ -21387,7 +21387,7 @@
         <v>36</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J77" s="2">
         <f>IF(I77&lt;&gt;"",I77,G77)</f>
@@ -21436,7 +21436,7 @@
         <v>28</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>106.59</v>
+        <v>189.5</v>
       </c>
       <c r="J78" s="2">
         <f>IF(I78&lt;&gt;"",I78,G78)</f>
@@ -21485,7 +21485,7 @@
         <v>30</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>10.35</v>
+        <v>18.4</v>
       </c>
       <c r="J79" s="2">
         <f>IF(I79&lt;&gt;"",I79,G79)</f>
@@ -21534,7 +21534,7 @@
         <v>28</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>10.35</v>
+        <v>18.4</v>
       </c>
       <c r="J80" s="2">
         <f>IF(I80&lt;&gt;"",I80,G80)</f>
@@ -21583,7 +21583,7 @@
         <v>26</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="J81" s="2">
         <f>IF(I81&lt;&gt;"",I81,G81)</f>
@@ -21632,7 +21632,7 @@
         <v>28</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J82" s="2">
         <f>IF(I82&lt;&gt;"",I82,G82)</f>
@@ -21681,7 +21681,7 @@
         <v>16</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>133.03</v>
+        <v>236.5</v>
       </c>
       <c r="J83" s="2">
         <f>IF(I83&lt;&gt;"",I83,G83)</f>
@@ -21730,7 +21730,7 @@
         <v>12</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>3.26</v>
+        <v>5.8</v>
       </c>
       <c r="J84" s="2">
         <f>IF(I84&lt;&gt;"",I84,G84)</f>
@@ -21779,7 +21779,7 @@
         <v>28</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>28.46</v>
+        <v>50.6</v>
       </c>
       <c r="J85" s="2">
         <f>IF(I85&lt;&gt;"",I85,G85)</f>
@@ -21828,7 +21828,7 @@
         <v>24</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>15.08</v>
+        <v>26.8</v>
       </c>
       <c r="J86" s="2">
         <f>IF(I86&lt;&gt;"",I86,G86)</f>
@@ -21877,7 +21877,7 @@
         <v>26</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>9.56</v>
+        <v>17</v>
       </c>
       <c r="J87" s="2">
         <f>IF(I87&lt;&gt;"",I87,G87)</f>
@@ -21926,7 +21926,7 @@
         <v>27</v>
       </c>
       <c r="I88" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="J88" s="2">
         <f>IF(I88&lt;&gt;"",I88,G88)</f>
@@ -21975,7 +21975,7 @@
         <v>24</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>19.01</v>
+        <v>33.8</v>
       </c>
       <c r="J89" s="2">
         <f>IF(I89&lt;&gt;"",I89,G89)</f>
@@ -22024,7 +22024,7 @@
         <v>21</v>
       </c>
       <c r="I90" s="3" t="n">
-        <v>19.8</v>
+        <v>35.2</v>
       </c>
       <c r="J90" s="2">
         <f>IF(I90&lt;&gt;"",I90,G90)</f>
@@ -22073,7 +22073,7 @@
         <v>27</v>
       </c>
       <c r="I91" s="3" t="n">
-        <v>7.99</v>
+        <v>14.2</v>
       </c>
       <c r="J91" s="2">
         <f>IF(I91&lt;&gt;"",I91,G91)</f>
@@ -22122,7 +22122,7 @@
         <v>27</v>
       </c>
       <c r="I92" s="3" t="n">
-        <v>7.99</v>
+        <v>14.2</v>
       </c>
       <c r="J92" s="2">
         <f>IF(I92&lt;&gt;"",I92,G92)</f>
@@ -22171,7 +22171,7 @@
         <v>18</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>44.51</v>
+        <v>79.13</v>
       </c>
       <c r="J93" s="2">
         <f>IF(I93&lt;&gt;"",I93,G93)</f>
@@ -22220,7 +22220,7 @@
         <v>30</v>
       </c>
       <c r="I94" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="J94" s="2">
         <f>IF(I94&lt;&gt;"",I94,G94)</f>
@@ -22269,7 +22269,7 @@
         <v>23</v>
       </c>
       <c r="I95" s="3" t="n">
-        <v>11.93</v>
+        <v>21.2</v>
       </c>
       <c r="J95" s="2">
         <f>IF(I95&lt;&gt;"",I95,G95)</f>
@@ -22318,7 +22318,7 @@
         <v>30</v>
       </c>
       <c r="I96" s="3" t="n">
-        <v>4.84</v>
+        <v>8.6</v>
       </c>
       <c r="J96" s="2">
         <f>IF(I96&lt;&gt;"",I96,G96)</f>
@@ -22367,7 +22367,7 @@
         <v>23</v>
       </c>
       <c r="I97" s="3" t="n">
-        <v>82.42</v>
+        <v>146.52</v>
       </c>
       <c r="J97" s="2">
         <f>IF(I97&lt;&gt;"",I97,G97)</f>
@@ -22416,7 +22416,7 @@
         <v>28</v>
       </c>
       <c r="I98" s="3" t="n">
-        <v>75.15000000000001</v>
+        <v>133.6</v>
       </c>
       <c r="J98" s="2">
         <f>IF(I98&lt;&gt;"",I98,G98)</f>
@@ -22465,7 +22465,7 @@
         <v>24</v>
       </c>
       <c r="I99" s="3" t="n">
-        <v>26.89</v>
+        <v>47.8</v>
       </c>
       <c r="J99" s="2">
         <f>IF(I99&lt;&gt;"",I99,G99)</f>
@@ -22514,7 +22514,7 @@
         <v>29</v>
       </c>
       <c r="I100" s="3" t="n">
-        <v>11.93</v>
+        <v>21.2</v>
       </c>
       <c r="J100" s="2">
         <f>IF(I100&lt;&gt;"",I100,G100)</f>
@@ -22563,7 +22563,7 @@
         <v>27</v>
       </c>
       <c r="I101" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J101" s="2">
         <f>IF(I101&lt;&gt;"",I101,G101)</f>
@@ -22612,7 +22612,7 @@
         <v>24</v>
       </c>
       <c r="I102" s="3" t="n">
-        <v>29.25</v>
+        <v>52</v>
       </c>
       <c r="J102" s="2">
         <f>IF(I102&lt;&gt;"",I102,G102)</f>
@@ -22661,7 +22661,7 @@
         <v>29</v>
       </c>
       <c r="I103" s="3" t="n">
-        <v>14.17</v>
+        <v>25.2</v>
       </c>
       <c r="J103" s="2">
         <f>IF(I103&lt;&gt;"",I103,G103)</f>
@@ -22710,7 +22710,7 @@
         <v>27</v>
       </c>
       <c r="I104" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="J104" s="2">
         <f>IF(I104&lt;&gt;"",I104,G104)</f>
@@ -22759,7 +22759,7 @@
         <v>27</v>
       </c>
       <c r="I105" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="J105" s="2">
         <f>IF(I105&lt;&gt;"",I105,G105)</f>
@@ -22808,7 +22808,7 @@
         <v>32</v>
       </c>
       <c r="I106" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="J106" s="2">
         <f>IF(I106&lt;&gt;"",I106,G106)</f>
@@ -22857,7 +22857,7 @@
         <v>30</v>
       </c>
       <c r="I107" s="3" t="n">
-        <v>9.56</v>
+        <v>17</v>
       </c>
       <c r="J107" s="2">
         <f>IF(I107&lt;&gt;"",I107,G107)</f>
@@ -22906,7 +22906,7 @@
         <v>27</v>
       </c>
       <c r="I108" s="3" t="n">
-        <v>4.84</v>
+        <v>8.6</v>
       </c>
       <c r="J108" s="2">
         <f>IF(I108&lt;&gt;"",I108,G108)</f>
@@ -22955,7 +22955,7 @@
         <v>29</v>
       </c>
       <c r="I109" s="3" t="n">
-        <v>14.96</v>
+        <v>26.6</v>
       </c>
       <c r="J109" s="2">
         <f>IF(I109&lt;&gt;"",I109,G109)</f>
@@ -23004,7 +23004,7 @@
         <v>30</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>7.99</v>
+        <v>14.2</v>
       </c>
       <c r="J110" s="2">
         <f>IF(I110&lt;&gt;"",I110,G110)</f>
@@ -23053,7 +23053,7 @@
         <v>25</v>
       </c>
       <c r="I111" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="J111" s="2">
         <f>IF(I111&lt;&gt;"",I111,G111)</f>
@@ -23102,7 +23102,7 @@
         <v>25</v>
       </c>
       <c r="I112" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="J112" s="2">
         <f>IF(I112&lt;&gt;"",I112,G112)</f>
@@ -23151,7 +23151,7 @@
         <v>26</v>
       </c>
       <c r="I113" s="3" t="n">
-        <v>55.8</v>
+        <v>99.2</v>
       </c>
       <c r="J113" s="2">
         <f>IF(I113&lt;&gt;"",I113,G113)</f>
@@ -23200,7 +23200,7 @@
         <v>32</v>
       </c>
       <c r="I114" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="J114" s="2">
         <f>IF(I114&lt;&gt;"",I114,G114)</f>
@@ -23249,7 +23249,7 @@
         <v>34</v>
       </c>
       <c r="I115" s="3" t="n">
-        <v>110.62</v>
+        <v>196.67</v>
       </c>
       <c r="J115" s="2">
         <f>IF(I115&lt;&gt;"",I115,G115)</f>
@@ -23298,7 +23298,7 @@
         <v>30</v>
       </c>
       <c r="I116" s="3" t="n">
-        <v>8.77</v>
+        <v>15.6</v>
       </c>
       <c r="J116" s="2">
         <f>IF(I116&lt;&gt;"",I116,G116)</f>
@@ -23347,7 +23347,7 @@
         <v>26</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="J117" s="2">
         <f>IF(I117&lt;&gt;"",I117,G117)</f>
@@ -23396,7 +23396,7 @@
         <v>28</v>
       </c>
       <c r="I118" s="3" t="n">
-        <v>171</v>
+        <v>304</v>
       </c>
       <c r="J118" s="2">
         <f>IF(I118&lt;&gt;"",I118,G118)</f>
@@ -23445,7 +23445,7 @@
         <v>29</v>
       </c>
       <c r="I119" s="3" t="n">
-        <v>26.1</v>
+        <v>46.4</v>
       </c>
       <c r="J119" s="2">
         <f>IF(I119&lt;&gt;"",I119,G119)</f>
@@ -23494,7 +23494,7 @@
         <v>28</v>
       </c>
       <c r="I120" s="3" t="n">
-        <v>12.71</v>
+        <v>22.6</v>
       </c>
       <c r="J120" s="2">
         <f>IF(I120&lt;&gt;"",I120,G120)</f>
@@ -23543,7 +23543,7 @@
         <v>34</v>
       </c>
       <c r="I121" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="J121" s="2">
         <f>IF(I121&lt;&gt;"",I121,G121)</f>
@@ -23592,7 +23592,7 @@
         <v>27</v>
       </c>
       <c r="I122" s="3" t="n">
-        <v>20.48</v>
+        <v>36.4</v>
       </c>
       <c r="J122" s="2">
         <f>IF(I122&lt;&gt;"",I122,G122)</f>
@@ -23641,7 +23641,7 @@
         <v>26</v>
       </c>
       <c r="I123" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="J123" s="2">
         <f>IF(I123&lt;&gt;"",I123,G123)</f>
@@ -23690,7 +23690,7 @@
         <v>25</v>
       </c>
       <c r="I124" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="J124" s="2">
         <f>IF(I124&lt;&gt;"",I124,G124)</f>
@@ -23739,7 +23739,7 @@
         <v>28</v>
       </c>
       <c r="I125" s="3" t="n">
-        <v>21.38</v>
+        <v>38</v>
       </c>
       <c r="J125" s="2">
         <f>IF(I125&lt;&gt;"",I125,G125)</f>
@@ -23788,7 +23788,7 @@
         <v>28</v>
       </c>
       <c r="I126" s="3" t="n">
-        <v>126.75</v>
+        <v>225.33</v>
       </c>
       <c r="J126" s="2">
         <f>IF(I126&lt;&gt;"",I126,G126)</f>
@@ -23837,7 +23837,7 @@
         <v>32</v>
       </c>
       <c r="I127" s="3" t="n">
-        <v>134.81</v>
+        <v>239.67</v>
       </c>
       <c r="J127" s="2">
         <f>IF(I127&lt;&gt;"",I127,G127)</f>
@@ -23886,7 +23886,7 @@
         <v>12</v>
       </c>
       <c r="I128" s="3" t="n">
-        <v>65.47</v>
+        <v>116.4</v>
       </c>
       <c r="J128" s="2">
         <f>IF(I128&lt;&gt;"",I128,G128)</f>
@@ -23935,7 +23935,7 @@
         <v>34</v>
       </c>
       <c r="I129" s="3" t="n">
-        <v>65.47</v>
+        <v>116.4</v>
       </c>
       <c r="J129" s="2">
         <f>IF(I129&lt;&gt;"",I129,G129)</f>
@@ -23984,7 +23984,7 @@
         <v>17</v>
       </c>
       <c r="I130" s="3" t="n">
-        <v>130.79</v>
+        <v>232.52</v>
       </c>
       <c r="J130" s="2">
         <f>IF(I130&lt;&gt;"",I130,G130)</f>
@@ -24033,7 +24033,7 @@
         <v>34</v>
       </c>
       <c r="I131" s="3" t="n">
-        <v>73.54000000000001</v>
+        <v>130.73</v>
       </c>
       <c r="J131" s="2">
         <f>IF(I131&lt;&gt;"",I131,G131)</f>
@@ -24082,7 +24082,7 @@
         <v>21</v>
       </c>
       <c r="I132" s="3" t="n">
-        <v>98.54000000000001</v>
+        <v>175.19</v>
       </c>
       <c r="J132" s="2">
         <f>IF(I132&lt;&gt;"",I132,G132)</f>
@@ -24131,7 +24131,7 @@
         <v>23</v>
       </c>
       <c r="I133" s="3" t="n">
-        <v>204</v>
+        <v>362.67</v>
       </c>
       <c r="J133" s="2">
         <f>IF(I133&lt;&gt;"",I133,G133)</f>
@@ -24180,7 +24180,7 @@
         <v>14</v>
       </c>
       <c r="I134" s="3" t="n">
-        <v>330</v>
+        <v>586.67</v>
       </c>
       <c r="J134" s="2">
         <f>IF(I134&lt;&gt;"",I134,G134)</f>
@@ -24229,7 +24229,7 @@
         <v>32</v>
       </c>
       <c r="I135" s="3" t="n">
-        <v>554.63</v>
+        <v>986</v>
       </c>
       <c r="J135" s="2">
         <f>IF(I135&lt;&gt;"",I135,G135)</f>
@@ -24278,7 +24278,7 @@
         <v>17</v>
       </c>
       <c r="I136" s="3" t="n">
-        <v>598.13</v>
+        <v>1063.33</v>
       </c>
       <c r="J136" s="2">
         <f>IF(I136&lt;&gt;"",I136,G136)</f>
@@ -24327,7 +24327,7 @@
         <v>29</v>
       </c>
       <c r="I137" s="3" t="n">
-        <v>556.88</v>
+        <v>990</v>
       </c>
       <c r="J137" s="2">
         <f>IF(I137&lt;&gt;"",I137,G137)</f>
@@ -24376,7 +24376,7 @@
         <v>22</v>
       </c>
       <c r="I138" s="3" t="n">
-        <v>556.88</v>
+        <v>990</v>
       </c>
       <c r="J138" s="2">
         <f>IF(I138&lt;&gt;"",I138,G138)</f>
@@ -24425,7 +24425,7 @@
         <v>17</v>
       </c>
       <c r="I139" s="3" t="n">
-        <v>595.88</v>
+        <v>1059.33</v>
       </c>
       <c r="J139" s="2">
         <f>IF(I139&lt;&gt;"",I139,G139)</f>
@@ -24474,7 +24474,7 @@
         <v>14</v>
       </c>
       <c r="I140" s="3" t="n">
-        <v>742.5</v>
+        <v>1320</v>
       </c>
       <c r="J140" s="2">
         <f>IF(I140&lt;&gt;"",I140,G140)</f>
@@ -24605,7 +24605,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>2145</v>
+        <v>3813.33</v>
       </c>
       <c r="I2" s="2">
         <f>IF(H2&lt;&gt;"",E2-H2,"")</f>
@@ -24642,7 +24642,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>866.25</v>
+        <v>1540</v>
       </c>
       <c r="I3" s="2">
         <f>IF(H3&lt;&gt;"",E3-H3,"")</f>
@@ -24679,7 +24679,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>657.75</v>
+        <v>1169.33</v>
       </c>
       <c r="I4" s="2">
         <f>IF(H4&lt;&gt;"",E4-H4,"")</f>
@@ -24716,7 +24716,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>616.5</v>
+        <v>1096</v>
       </c>
       <c r="I5" s="2">
         <f>IF(H5&lt;&gt;"",E5-H5,"")</f>
@@ -24753,7 +24753,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>577.5</v>
+        <v>1026.67</v>
       </c>
       <c r="I6" s="2">
         <f>IF(H6&lt;&gt;"",E6-H6,"")</f>
@@ -24790,7 +24790,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>453.75</v>
+        <v>806.67</v>
       </c>
       <c r="I7" s="2">
         <f>IF(H7&lt;&gt;"",E7-H7,"")</f>
@@ -24827,7 +24827,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>379.5</v>
+        <v>674.67</v>
       </c>
       <c r="I8" s="2">
         <f>IF(H8&lt;&gt;"",E8-H8,"")</f>
@@ -24864,7 +24864,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>261.75</v>
+        <v>465.33</v>
       </c>
       <c r="I9" s="2">
         <f>IF(H9&lt;&gt;"",E9-H9,"")</f>
@@ -24901,7 +24901,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>261.75</v>
+        <v>465.33</v>
       </c>
       <c r="I10" s="2">
         <f>IF(H10&lt;&gt;"",E10-H10,"")</f>
@@ -24938,7 +24938,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>253.5</v>
+        <v>450.67</v>
       </c>
       <c r="I11" s="2">
         <f>IF(H11&lt;&gt;"",E11-H11,"")</f>
@@ -24975,7 +24975,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>228.75</v>
+        <v>406.67</v>
       </c>
       <c r="I12" s="2">
         <f>IF(H12&lt;&gt;"",E12-H12,"")</f>
@@ -25012,7 +25012,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>214.5</v>
+        <v>381.33</v>
       </c>
       <c r="I13" s="2">
         <f>IF(H13&lt;&gt;"",E13-H13,"")</f>
@@ -25049,7 +25049,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>179.25</v>
+        <v>318.67</v>
       </c>
       <c r="I14" s="2">
         <f>IF(H14&lt;&gt;"",E14-H14,"")</f>
@@ -25086,7 +25086,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>173.25</v>
+        <v>308</v>
       </c>
       <c r="I15" s="2">
         <f>IF(H15&lt;&gt;"",E15-H15,"")</f>
@@ -25123,7 +25123,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>162.75</v>
+        <v>289.33</v>
       </c>
       <c r="I16" s="2">
         <f>IF(H16&lt;&gt;"",E16-H16,"")</f>
@@ -25160,7 +25160,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>141.09</v>
+        <v>250.83</v>
       </c>
       <c r="I17" s="2">
         <f>IF(H17&lt;&gt;"",E17-H17,"")</f>
@@ -25197,7 +25197,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>133.03</v>
+        <v>236.5</v>
       </c>
       <c r="I18" s="2">
         <f>IF(H18&lt;&gt;"",E18-H18,"")</f>
@@ -25234,7 +25234,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>126.75</v>
+        <v>225.33</v>
       </c>
       <c r="I19" s="2">
         <f>IF(H19&lt;&gt;"",E19-H19,"")</f>
@@ -25271,7 +25271,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>102.56</v>
+        <v>182.33</v>
       </c>
       <c r="I20" s="2">
         <f>IF(H20&lt;&gt;"",E20-H20,"")</f>
@@ -25308,7 +25308,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>98.53</v>
+        <v>175.17</v>
       </c>
       <c r="I21" s="2">
         <f>IF(H21&lt;&gt;"",E21-H21,"")</f>
@@ -25345,7 +25345,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>90.48</v>
+        <v>160.85</v>
       </c>
       <c r="I22" s="2">
         <f>IF(H22&lt;&gt;"",E22-H22,"")</f>
@@ -25382,7 +25382,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>86.44</v>
+        <v>153.67</v>
       </c>
       <c r="I23" s="2">
         <f>IF(H23&lt;&gt;"",E23-H23,"")</f>
@@ -25419,7 +25419,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>78.38</v>
+        <v>139.33</v>
       </c>
       <c r="I24" s="2">
         <f>IF(H24&lt;&gt;"",E24-H24,"")</f>
@@ -25456,7 +25456,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>70.31</v>
+        <v>125</v>
       </c>
       <c r="I25" s="2">
         <f>IF(H25&lt;&gt;"",E25-H25,"")</f>
@@ -25493,7 +25493,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>68.7</v>
+        <v>122.13</v>
       </c>
       <c r="I26" s="2">
         <f>IF(H26&lt;&gt;"",E26-H26,"")</f>
@@ -25530,7 +25530,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>68.7</v>
+        <v>122.13</v>
       </c>
       <c r="I27" s="2">
         <f>IF(H27&lt;&gt;"",E27-H27,"")</f>
@@ -25567,7 +25567,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>68.7</v>
+        <v>122.13</v>
       </c>
       <c r="I28" s="2">
         <f>IF(H28&lt;&gt;"",E28-H28,"")</f>
@@ -25604,7 +25604,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>65.47</v>
+        <v>116.4</v>
       </c>
       <c r="I29" s="2">
         <f>IF(H29&lt;&gt;"",E29-H29,"")</f>
@@ -25641,7 +25641,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>63.86</v>
+        <v>113.53</v>
       </c>
       <c r="I30" s="2">
         <f>IF(H30&lt;&gt;"",E30-H30,"")</f>
@@ -25678,7 +25678,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>59.66</v>
+        <v>106.07</v>
       </c>
       <c r="I31" s="2">
         <f>IF(H31&lt;&gt;"",E31-H31,"")</f>
@@ -25715,7 +25715,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>55.8</v>
+        <v>99.2</v>
       </c>
       <c r="I32" s="2">
         <f>IF(H32&lt;&gt;"",E32-H32,"")</f>
@@ -25752,7 +25752,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>54.19</v>
+        <v>96.33</v>
       </c>
       <c r="I33" s="2">
         <f>IF(H33&lt;&gt;"",E33-H33,"")</f>
@@ -25789,7 +25789,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>52.57</v>
+        <v>93.47</v>
       </c>
       <c r="I34" s="2">
         <f>IF(H34&lt;&gt;"",E34-H34,"")</f>
@@ -25826,7 +25826,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>52.57</v>
+        <v>93.47</v>
       </c>
       <c r="I35" s="2">
         <f>IF(H35&lt;&gt;"",E35-H35,"")</f>
@@ -25863,7 +25863,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>50.96</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="I36" s="2">
         <f>IF(H36&lt;&gt;"",E36-H36,"")</f>
@@ -25900,7 +25900,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>49.99</v>
+        <v>88.87</v>
       </c>
       <c r="I37" s="2">
         <f>IF(H37&lt;&gt;"",E37-H37,"")</f>
@@ -25937,7 +25937,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>49.35</v>
+        <v>87.73</v>
       </c>
       <c r="I38" s="2">
         <f>IF(H38&lt;&gt;"",E38-H38,"")</f>
@@ -25974,7 +25974,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>48.15</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="I39" s="2">
         <f>IF(H39&lt;&gt;"",E39-H39,"")</f>
@@ -26011,7 +26011,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>47.74</v>
+        <v>84.87</v>
       </c>
       <c r="I40" s="2">
         <f>IF(H40&lt;&gt;"",E40-H40,"")</f>
@@ -26048,7 +26048,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>46.12</v>
+        <v>82</v>
       </c>
       <c r="I41" s="2">
         <f>IF(H41&lt;&gt;"",E41-H41,"")</f>
@@ -26085,7 +26085,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>39.67</v>
+        <v>70.53</v>
       </c>
       <c r="I42" s="2">
         <f>IF(H42&lt;&gt;"",E42-H42,"")</f>
@@ -26122,7 +26122,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>39.67</v>
+        <v>70.53</v>
       </c>
       <c r="I43" s="2">
         <f>IF(H43&lt;&gt;"",E43-H43,"")</f>
@@ -26159,7 +26159,7 @@
         <v>0</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>39.67</v>
+        <v>70.53</v>
       </c>
       <c r="I44" s="2">
         <f>IF(H44&lt;&gt;"",E44-H44,"")</f>
@@ -26196,7 +26196,7 @@
         <v>0</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>38.06</v>
+        <v>67.67</v>
       </c>
       <c r="I45" s="2">
         <f>IF(H45&lt;&gt;"",E45-H45,"")</f>
@@ -26233,7 +26233,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>36.34</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="I46" s="2">
         <f>IF(H46&lt;&gt;"",E46-H46,"")</f>
@@ -26270,7 +26270,7 @@
         <v>0</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>35.44</v>
+        <v>63</v>
       </c>
       <c r="I47" s="2">
         <f>IF(H47&lt;&gt;"",E47-H47,"")</f>
@@ -26307,7 +26307,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>33.97</v>
+        <v>60.4</v>
       </c>
       <c r="I48" s="2">
         <f>IF(H48&lt;&gt;"",E48-H48,"")</f>
@@ -26344,7 +26344,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>33.19</v>
+        <v>59</v>
       </c>
       <c r="I49" s="2">
         <f>IF(H49&lt;&gt;"",E49-H49,"")</f>
@@ -26381,7 +26381,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>33.19</v>
+        <v>59</v>
       </c>
       <c r="I50" s="2">
         <f>IF(H50&lt;&gt;"",E50-H50,"")</f>
@@ -26418,7 +26418,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>32.4</v>
+        <v>57.6</v>
       </c>
       <c r="I51" s="2">
         <f>IF(H51&lt;&gt;"",E51-H51,"")</f>
@@ -26455,7 +26455,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>30.04</v>
+        <v>53.4</v>
       </c>
       <c r="I52" s="2">
         <f>IF(H52&lt;&gt;"",E52-H52,"")</f>
@@ -26492,7 +26492,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>30.04</v>
+        <v>53.4</v>
       </c>
       <c r="I53" s="2">
         <f>IF(H53&lt;&gt;"",E53-H53,"")</f>
@@ -26529,7 +26529,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>26.89</v>
+        <v>47.8</v>
       </c>
       <c r="I54" s="2">
         <f>IF(H54&lt;&gt;"",E54-H54,"")</f>
@@ -26566,7 +26566,7 @@
         <v>0</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>26.1</v>
+        <v>46.4</v>
       </c>
       <c r="I55" s="2">
         <f>IF(H55&lt;&gt;"",E55-H55,"")</f>
@@ -26603,7 +26603,7 @@
         <v>0</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>25.31</v>
+        <v>45</v>
       </c>
       <c r="I56" s="2">
         <f>IF(H56&lt;&gt;"",E56-H56,"")</f>
@@ -26640,7 +26640,7 @@
         <v>0</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>24.53</v>
+        <v>43.6</v>
       </c>
       <c r="I57" s="2">
         <f>IF(H57&lt;&gt;"",E57-H57,"")</f>
@@ -26677,7 +26677,7 @@
         <v>0</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>24.41</v>
+        <v>43.4</v>
       </c>
       <c r="I58" s="2">
         <f>IF(H58&lt;&gt;"",E58-H58,"")</f>
@@ -26714,7 +26714,7 @@
         <v>0</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>23.74</v>
+        <v>42.2</v>
       </c>
       <c r="I59" s="2">
         <f>IF(H59&lt;&gt;"",E59-H59,"")</f>
@@ -26751,7 +26751,7 @@
         <v>0</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>22.16</v>
+        <v>39.4</v>
       </c>
       <c r="I60" s="2">
         <f>IF(H60&lt;&gt;"",E60-H60,"")</f>
@@ -26788,7 +26788,7 @@
         <v>0</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>22.16</v>
+        <v>39.4</v>
       </c>
       <c r="I61" s="2">
         <f>IF(H61&lt;&gt;"",E61-H61,"")</f>
@@ -26825,7 +26825,7 @@
         <v>0</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>20.59</v>
+        <v>36.6</v>
       </c>
       <c r="I62" s="2">
         <f>IF(H62&lt;&gt;"",E62-H62,"")</f>
@@ -26862,7 +26862,7 @@
         <v>0</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>20.59</v>
+        <v>36.6</v>
       </c>
       <c r="I63" s="2">
         <f>IF(H63&lt;&gt;"",E63-H63,"")</f>
@@ -26899,7 +26899,7 @@
         <v>0</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>18.23</v>
+        <v>32.4</v>
       </c>
       <c r="I64" s="2">
         <f>IF(H64&lt;&gt;"",E64-H64,"")</f>
@@ -26936,7 +26936,7 @@
         <v>0</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>18.23</v>
+        <v>32.4</v>
       </c>
       <c r="I65" s="2">
         <f>IF(H65&lt;&gt;"",E65-H65,"")</f>
@@ -26973,7 +26973,7 @@
         <v>0</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>15.08</v>
+        <v>26.8</v>
       </c>
       <c r="I66" s="2">
         <f>IF(H66&lt;&gt;"",E66-H66,"")</f>
@@ -27010,7 +27010,7 @@
         <v>0</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>14.29</v>
+        <v>25.4</v>
       </c>
       <c r="I67" s="2">
         <f>IF(H67&lt;&gt;"",E67-H67,"")</f>
@@ -27047,7 +27047,7 @@
         <v>0</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>13.5</v>
+        <v>24</v>
       </c>
       <c r="I68" s="2">
         <f>IF(H68&lt;&gt;"",E68-H68,"")</f>
@@ -27084,7 +27084,7 @@
         <v>0</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>13.5</v>
+        <v>24</v>
       </c>
       <c r="I69" s="2">
         <f>IF(H69&lt;&gt;"",E69-H69,"")</f>
@@ -27121,7 +27121,7 @@
         <v>0</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>12.71</v>
+        <v>22.6</v>
       </c>
       <c r="I70" s="2">
         <f>IF(H70&lt;&gt;"",E70-H70,"")</f>
@@ -27158,7 +27158,7 @@
         <v>0</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>12.6</v>
+        <v>22.4</v>
       </c>
       <c r="I71" s="2">
         <f>IF(H71&lt;&gt;"",E71-H71,"")</f>
@@ -27195,7 +27195,7 @@
         <v>0</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>11.93</v>
+        <v>21.2</v>
       </c>
       <c r="I72" s="2">
         <f>IF(H72&lt;&gt;"",E72-H72,"")</f>
@@ -27232,7 +27232,7 @@
         <v>0</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>11.14</v>
+        <v>19.8</v>
       </c>
       <c r="I73" s="2">
         <f>IF(H73&lt;&gt;"",E73-H73,"")</f>
@@ -27269,7 +27269,7 @@
         <v>0</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>11.14</v>
+        <v>19.8</v>
       </c>
       <c r="I74" s="2">
         <f>IF(H74&lt;&gt;"",E74-H74,"")</f>
@@ -27306,7 +27306,7 @@
         <v>0</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>10.35</v>
+        <v>18.4</v>
       </c>
       <c r="I75" s="2">
         <f>IF(H75&lt;&gt;"",E75-H75,"")</f>
@@ -27343,7 +27343,7 @@
         <v>0</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>9.56</v>
+        <v>17</v>
       </c>
       <c r="I76" s="2">
         <f>IF(H76&lt;&gt;"",E76-H76,"")</f>
@@ -27380,7 +27380,7 @@
         <v>0</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>8.77</v>
+        <v>15.6</v>
       </c>
       <c r="I77" s="2">
         <f>IF(H77&lt;&gt;"",E77-H77,"")</f>
@@ -27417,7 +27417,7 @@
         <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>7.99</v>
+        <v>14.2</v>
       </c>
       <c r="I78" s="2">
         <f>IF(H78&lt;&gt;"",E78-H78,"")</f>
@@ -27454,7 +27454,7 @@
         <v>0</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>7.2</v>
+        <v>12.8</v>
       </c>
       <c r="I79" s="2">
         <f>IF(H79&lt;&gt;"",E79-H79,"")</f>
@@ -27491,7 +27491,7 @@
         <v>0</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="I80" s="2">
         <f>IF(H80&lt;&gt;"",E80-H80,"")</f>
@@ -27528,7 +27528,7 @@
         <v>0</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="I81" s="2">
         <f>IF(H81&lt;&gt;"",E81-H81,"")</f>
@@ -27565,7 +27565,7 @@
         <v>0</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>6.41</v>
+        <v>11.4</v>
       </c>
       <c r="I82" s="2">
         <f>IF(H82&lt;&gt;"",E82-H82,"")</f>
@@ -27602,7 +27602,7 @@
         <v>0</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="I83" s="2">
         <f>IF(H83&lt;&gt;"",E83-H83,"")</f>
@@ -27639,7 +27639,7 @@
         <v>0</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>5.62</v>
+        <v>10</v>
       </c>
       <c r="I84" s="2">
         <f>IF(H84&lt;&gt;"",E84-H84,"")</f>
@@ -27676,7 +27676,7 @@
         <v>0</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I85" s="2">
         <f>IF(H85&lt;&gt;"",E85-H85,"")</f>
@@ -27713,7 +27713,7 @@
         <v>0</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I86" s="2">
         <f>IF(H86&lt;&gt;"",E86-H86,"")</f>
@@ -27750,7 +27750,7 @@
         <v>0</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I87" s="2">
         <f>IF(H87&lt;&gt;"",E87-H87,"")</f>
@@ -27787,7 +27787,7 @@
         <v>0</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I88" s="2">
         <f>IF(H88&lt;&gt;"",E88-H88,"")</f>
@@ -27824,7 +27824,7 @@
         <v>0</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I89" s="2">
         <f>IF(H89&lt;&gt;"",E89-H89,"")</f>
@@ -27861,7 +27861,7 @@
         <v>0</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>4.05</v>
+        <v>7.2</v>
       </c>
       <c r="I90" s="2">
         <f>IF(H90&lt;&gt;"",E90-H90,"")</f>
@@ -27898,7 +27898,7 @@
         <v>0</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="I91" s="2">
         <f>IF(H91&lt;&gt;"",E91-H91,"")</f>
@@ -27935,7 +27935,7 @@
         <v>0</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>2.48</v>
+        <v>4.4</v>
       </c>
       <c r="I92" s="2">
         <f>IF(H92&lt;&gt;"",E92-H92,"")</f>
@@ -27972,7 +27972,7 @@
         <v>0</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="I93" s="2">
         <f>IF(H93&lt;&gt;"",E93-H93,"")</f>
@@ -28009,7 +28009,7 @@
         <v>0</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>1.69</v>
+        <v>3</v>
       </c>
       <c r="I94" s="2">
         <f>IF(H94&lt;&gt;"",E94-H94,"")</f>
@@ -28020,6 +28020,7 @@
         <v/>
       </c>
     </row>
+    <row r="95"/>
     <row r="96">
       <c r="D96" s="1" t="inlineStr">
         <is>

</xml_diff>